<commit_message>
Added day 2 NPC decks
</commit_message>
<xml_diff>
--- a/Coin_tracker.xlsx
+++ b/Coin_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{930A508A-D596-4EE0-B55B-91D8F955D65A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2984F12C-AD05-4F26-AC69-3581BF6260E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25335" yWindow="2235" windowWidth="43200" windowHeight="11835" xr2:uid="{2902C7A9-D4C7-4F9F-B9D2-2E43E3BE476A}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="28800" windowHeight="17685" xr2:uid="{2902C7A9-D4C7-4F9F-B9D2-2E43E3BE476A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="188">
   <si>
     <t>coin_alakazam_purple.png</t>
   </si>
@@ -597,6 +597,9 @@
   </si>
   <si>
     <t>jericho eve 1</t>
+  </si>
+  <si>
+    <t>kenneth day 2</t>
   </si>
 </sst>
 </file>
@@ -992,6 +995,9 @@
       <c r="A3" t="s">
         <v>1</v>
       </c>
+      <c r="B3" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">

</xml_diff>

<commit_message>
Finished most of day evening and night 2 NPC and Opponents
</commit_message>
<xml_diff>
--- a/Coin_tracker.xlsx
+++ b/Coin_tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2984F12C-AD05-4F26-AC69-3581BF6260E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DF0F8A0-2BF1-422A-BD90-052870D427C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="28800" windowHeight="17685" xr2:uid="{2902C7A9-D4C7-4F9F-B9D2-2E43E3BE476A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{2902C7A9-D4C7-4F9F-B9D2-2E43E3BE476A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="207">
   <si>
     <t>coin_alakazam_purple.png</t>
   </si>
@@ -572,34 +572,91 @@
     <t>Coin</t>
   </si>
   <si>
-    <t>granted by</t>
-  </si>
-  <si>
-    <t>joey day 1</t>
-  </si>
-  <si>
-    <t>mick day 1</t>
-  </si>
-  <si>
-    <t>adam day 1</t>
-  </si>
-  <si>
-    <t>dave day 1</t>
-  </si>
-  <si>
-    <t>callum eve 1</t>
-  </si>
-  <si>
-    <t>allan eve 1</t>
-  </si>
-  <si>
-    <t>john eve 1</t>
-  </si>
-  <si>
-    <t>jericho eve 1</t>
-  </si>
-  <si>
-    <t>kenneth day 2</t>
+    <t>Birdspotter_Tamsin</t>
+  </si>
+  <si>
+    <t>granted by name</t>
+  </si>
+  <si>
+    <t>granted day</t>
+  </si>
+  <si>
+    <t>Day 2</t>
+  </si>
+  <si>
+    <t>Firebreather Kenneth</t>
+  </si>
+  <si>
+    <t>Gardener Callum</t>
+  </si>
+  <si>
+    <t>Evening 1</t>
+  </si>
+  <si>
+    <t>Schoolboy_Adam</t>
+  </si>
+  <si>
+    <t>Day 1</t>
+  </si>
+  <si>
+    <t>Painter Jericho</t>
+  </si>
+  <si>
+    <t>Youngster Joey</t>
+  </si>
+  <si>
+    <t>Engineer Allan</t>
+  </si>
+  <si>
+    <t>Fisherman Dave</t>
+  </si>
+  <si>
+    <t>Fisherman John</t>
+  </si>
+  <si>
+    <t>Gambler Mick</t>
+  </si>
+  <si>
+    <t>Swimmer Jordan</t>
+  </si>
+  <si>
+    <t>Swimmer Todd</t>
+  </si>
+  <si>
+    <t>Battlegirl Sofia</t>
+  </si>
+  <si>
+    <t>Sailor Bob</t>
+  </si>
+  <si>
+    <t>Bug Catcher Johnny</t>
+  </si>
+  <si>
+    <t>Bug Catcher Alex</t>
+  </si>
+  <si>
+    <t>Psychic Brienne</t>
+  </si>
+  <si>
+    <t>FireBreather Darryl</t>
+  </si>
+  <si>
+    <t>Beach Kid Evie</t>
+  </si>
+  <si>
+    <t>Beach Kid Timothy</t>
+  </si>
+  <si>
+    <t>Sunbathing coin giver</t>
+  </si>
+  <si>
+    <t>Jogger Daniel</t>
+  </si>
+  <si>
+    <t>Evening 2</t>
+  </si>
+  <si>
+    <t>Bad Dude Paul</t>
   </si>
 </sst>
 </file>
@@ -971,350 +1028,426 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E36B1B59-0D5E-4C8D-AEE2-CA809DBB4E7C}">
-  <dimension ref="A1:B178"/>
+  <dimension ref="A1:C178"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>177</v>
       </c>
       <c r="B1" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+      <c r="C1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+      <c r="C3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
       <c r="B9" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+      <c r="C13" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>178</v>
+      </c>
+      <c r="C21" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>33</v>
       </c>
-      <c r="B35" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>187</v>
+      </c>
+      <c r="C44" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>193</v>
+      </c>
+      <c r="C48" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>194</v>
+      </c>
+      <c r="C49" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>195</v>
+      </c>
+      <c r="C50" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>196</v>
+      </c>
+      <c r="C51" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>50</v>
       </c>
       <c r="B52" t="s">
+        <v>189</v>
+      </c>
+      <c r="C52" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>198</v>
+      </c>
+      <c r="C55" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>197</v>
+      </c>
+      <c r="C56" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>199</v>
+      </c>
+      <c r="C58" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>200</v>
+      </c>
+      <c r="C60" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+      <c r="C63" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>62</v>
       </c>
@@ -1399,491 +1532,530 @@
         <v>78</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+      <c r="C82" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>81</v>
       </c>
       <c r="B83" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+      <c r="C83" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B105" t="s">
+        <v>201</v>
+      </c>
+      <c r="C105" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>121</v>
       </c>
       <c r="B123" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+      <c r="C123" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
+        <v>202</v>
+      </c>
+      <c r="C125" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B140" t="s">
+        <v>206</v>
+      </c>
+      <c r="C140" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B145" t="s">
+        <v>204</v>
+      </c>
+      <c r="C145" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B174" t="s">
+        <v>203</v>
+      </c>
+      <c r="C174" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>174</v>
       </c>

</xml_diff>

<commit_message>
Finished most of day and some of evening 3 NPC/Opponents
</commit_message>
<xml_diff>
--- a/Coin_tracker.xlsx
+++ b/Coin_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DF0F8A0-2BF1-422A-BD90-052870D427C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDD1781-6DB5-4E36-A2AF-8A9C02A852E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{2902C7A9-D4C7-4F9F-B9D2-2E43E3BE476A}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17280" xr2:uid="{2902C7A9-D4C7-4F9F-B9D2-2E43E3BE476A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="224">
   <si>
     <t>coin_alakazam_purple.png</t>
   </si>
@@ -572,9 +572,6 @@
     <t>Coin</t>
   </si>
   <si>
-    <t>Birdspotter_Tamsin</t>
-  </si>
-  <si>
     <t>granted by name</t>
   </si>
   <si>
@@ -657,14 +654,76 @@
   </si>
   <si>
     <t>Bad Dude Paul</t>
+  </si>
+  <si>
+    <t>Coin Shop</t>
+  </si>
+  <si>
+    <t>Day 3+</t>
+  </si>
+  <si>
+    <t>Juice Bar</t>
+  </si>
+  <si>
+    <t>Day 2+</t>
+  </si>
+  <si>
+    <t>Day 3</t>
+  </si>
+  <si>
+    <t>Birdspotter Gregg</t>
+  </si>
+  <si>
+    <t>Swimmer Melissa</t>
+  </si>
+  <si>
+    <t>Bug Catcher Frankie</t>
+  </si>
+  <si>
+    <t>coin_gyarados_gold.png</t>
+  </si>
+  <si>
+    <t>Fisherman Gary</t>
+  </si>
+  <si>
+    <t>SS Anne Tourist Edmund</t>
+  </si>
+  <si>
+    <t>SS Anne Tourist Alissa</t>
+  </si>
+  <si>
+    <t>Guitarist Jonesy</t>
+  </si>
+  <si>
+    <t>Birdspotter Tamsin</t>
+  </si>
+  <si>
+    <t>Guitarist Howard</t>
+  </si>
+  <si>
+    <t>Young Twin Nella</t>
+  </si>
+  <si>
+    <t>Young Twin Anna</t>
+  </si>
+  <si>
+    <t>Garden Manager Louis</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -692,13 +751,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -709,6 +788,21 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CABA093D-E10D-4AFA-84B7-B1B7EB5F6B16}" name="Table1" displayName="Table1" ref="A1:C179" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:C179" xr:uid="{CABA093D-E10D-4AFA-84B7-B1B7EB5F6B16}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C177">
+    <sortCondition ref="B1:B179"/>
+  </sortState>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{B1B3F4BF-11CF-4DCD-BBFF-800CA95AB652}" name="Coin"/>
+    <tableColumn id="2" xr3:uid="{2B45EC9D-2894-4946-81C0-66214EF570D9}" name="granted by name"/>
+    <tableColumn id="3" xr3:uid="{7746DE0B-7B46-4C19-BAE4-2167203617DB}" name="granted day"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1028,23 +1122,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E36B1B59-0D5E-4C8D-AEE2-CA809DBB4E7C}">
-  <dimension ref="A1:C178"/>
+  <dimension ref="A1:C179"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.28515625" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="C1" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1057,16 +1151,22 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
+      <c r="B4" t="s">
+        <v>206</v>
+      </c>
+      <c r="C4" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -1093,10 +1193,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" t="s">
         <v>183</v>
-      </c>
-      <c r="C9" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1108,21 +1208,33 @@
       <c r="A11" t="s">
         <v>9</v>
       </c>
+      <c r="B11" t="s">
+        <v>222</v>
+      </c>
+      <c r="C11" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
+      <c r="B12" t="s">
+        <v>221</v>
+      </c>
+      <c r="C12" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
       <c r="B13" t="s">
+        <v>184</v>
+      </c>
+      <c r="C13" t="s">
         <v>185</v>
-      </c>
-      <c r="C13" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1165,10 +1277,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>178</v>
+        <v>219</v>
       </c>
       <c r="C21" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1245,6 +1357,9 @@
       <c r="A36" t="s">
         <v>34</v>
       </c>
+      <c r="B36" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
@@ -1286,10 +1401,10 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C44" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1312,10 +1427,10 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C48" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1323,10 +1438,10 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C49" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1334,10 +1449,10 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C50" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1345,10 +1460,10 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C51" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1356,10 +1471,10 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C52" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1377,21 +1492,18 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C55" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>54</v>
       </c>
-      <c r="B56" t="s">
-        <v>197</v>
-      </c>
       <c r="C56" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -1404,10 +1516,10 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C58" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -1420,10 +1532,10 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -1441,10 +1553,10 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C63" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -1452,82 +1564,94 @@
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
+        <v>206</v>
+      </c>
+      <c r="C75" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B76" t="s">
+        <v>213</v>
+      </c>
+      <c r="C76" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>78</v>
       </c>
@@ -1542,535 +1666,648 @@
         <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C82" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>81</v>
+        <v>214</v>
       </c>
       <c r="B83" t="s">
-        <v>191</v>
+        <v>215</v>
       </c>
       <c r="C83" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>82</v>
+        <v>81</v>
+      </c>
+      <c r="B84" t="s">
+        <v>190</v>
+      </c>
+      <c r="C84" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>83</v>
+        <v>82</v>
+      </c>
+      <c r="B85" t="s">
+        <v>206</v>
+      </c>
+      <c r="C85" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>85</v>
+        <v>84</v>
+      </c>
+      <c r="B87" t="s">
+        <v>217</v>
+      </c>
+      <c r="C87" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>89</v>
+        <v>88</v>
+      </c>
+      <c r="B91" t="s">
+        <v>212</v>
+      </c>
+      <c r="C91" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>94</v>
+        <v>93</v>
+      </c>
+      <c r="B96" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>103</v>
-      </c>
-      <c r="B105" t="s">
-        <v>201</v>
-      </c>
-      <c r="C105" t="s">
-        <v>181</v>
+        <v>102</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="B106" t="s">
+        <v>200</v>
+      </c>
+      <c r="C106" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>106</v>
+        <v>105</v>
+      </c>
+      <c r="C108" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>108</v>
+        <v>107</v>
+      </c>
+      <c r="B110" t="s">
+        <v>208</v>
+      </c>
+      <c r="C110" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>109</v>
+        <v>108</v>
+      </c>
+      <c r="B111" t="s">
+        <v>208</v>
+      </c>
+      <c r="C111" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>118</v>
+        <v>117</v>
+      </c>
+      <c r="B120" t="s">
+        <v>206</v>
+      </c>
+      <c r="C120" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>121</v>
-      </c>
-      <c r="B123" t="s">
-        <v>192</v>
-      </c>
-      <c r="C123" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>122</v>
+        <v>121</v>
+      </c>
+      <c r="B124" t="s">
+        <v>191</v>
+      </c>
+      <c r="C124" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>123</v>
-      </c>
-      <c r="B125" t="s">
-        <v>202</v>
-      </c>
-      <c r="C125" t="s">
-        <v>181</v>
+        <v>122</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>124</v>
+        <v>123</v>
+      </c>
+      <c r="B126" t="s">
+        <v>201</v>
+      </c>
+      <c r="C126" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>138</v>
-      </c>
-      <c r="B140" t="s">
-        <v>206</v>
-      </c>
-      <c r="C140" t="s">
-        <v>205</v>
+        <v>137</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>139</v>
+        <v>138</v>
+      </c>
+      <c r="B141" t="s">
+        <v>205</v>
+      </c>
+      <c r="C141" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>143</v>
-      </c>
-      <c r="B145" t="s">
-        <v>204</v>
-      </c>
-      <c r="C145" t="s">
-        <v>205</v>
+        <v>142</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>144</v>
+        <v>143</v>
+      </c>
+      <c r="B146" t="s">
+        <v>203</v>
+      </c>
+      <c r="C146" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>149</v>
+        <v>148</v>
+      </c>
+      <c r="B151" t="s">
+        <v>220</v>
+      </c>
+      <c r="C151" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>155</v>
+        <v>154</v>
+      </c>
+      <c r="B157" t="s">
+        <v>206</v>
+      </c>
+      <c r="C157" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>159</v>
+        <v>158</v>
+      </c>
+      <c r="B161" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>165</v>
+        <v>164</v>
+      </c>
+      <c r="B167" t="s">
+        <v>206</v>
+      </c>
+      <c r="C167" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>166</v>
+        <v>165</v>
+      </c>
+      <c r="B168" t="s">
+        <v>206</v>
+      </c>
+      <c r="C168" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>168</v>
+        <v>167</v>
+      </c>
+      <c r="B170" t="s">
+        <v>223</v>
+      </c>
+      <c r="C170" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>170</v>
+        <v>169</v>
+      </c>
+      <c r="B172" t="s">
+        <v>206</v>
+      </c>
+      <c r="C172" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B174" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C174" t="s">
-        <v>181</v>
+        <v>207</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>173</v>
+        <v>172</v>
+      </c>
+      <c r="B175" t="s">
+        <v>202</v>
+      </c>
+      <c r="C175" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A177" t="s">
+      <c r="B177" t="s">
+        <v>206</v>
+      </c>
+      <c r="C177" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A178" t="s">
+      <c r="B178" t="s">
+        <v>218</v>
+      </c>
+      <c r="C178" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
         <v>176</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finished most if not all of day, evening and night 3 opponents and npcs
</commit_message>
<xml_diff>
--- a/Coin_tracker.xlsx
+++ b/Coin_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDD1781-6DB5-4E36-A2AF-8A9C02A852E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD2F134-986D-4142-84C3-B6881BF76845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17280" xr2:uid="{2902C7A9-D4C7-4F9F-B9D2-2E43E3BE476A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{2902C7A9-D4C7-4F9F-B9D2-2E43E3BE476A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="415">
   <si>
     <t>coin_alakazam_purple.png</t>
   </si>
@@ -518,9 +518,6 @@
     <t>coin_tyranitar_blue.png</t>
   </si>
   <si>
-    <t>coin_tyranitar_gold_2.png</t>
-  </si>
-  <si>
     <t>coin_tyranitar_silver.png</t>
   </si>
   <si>
@@ -708,6 +705,582 @@
   </si>
   <si>
     <t>Garden Manager Louis</t>
+  </si>
+  <si>
+    <t>Card Elder Rayne</t>
+  </si>
+  <si>
+    <t>Day 3-4</t>
+  </si>
+  <si>
+    <t>Card Elder Waverly</t>
+  </si>
+  <si>
+    <t>Card Elder Hamish</t>
+  </si>
+  <si>
+    <t>coin_tyranitar_gold.png</t>
+  </si>
+  <si>
+    <t>Coin Name</t>
+  </si>
+  <si>
+    <t>alakazam purple</t>
+  </si>
+  <si>
+    <t>arcanine red</t>
+  </si>
+  <si>
+    <t>arceus silver</t>
+  </si>
+  <si>
+    <t>back basic</t>
+  </si>
+  <si>
+    <t>blastoise blue</t>
+  </si>
+  <si>
+    <t>blastoise blue 2</t>
+  </si>
+  <si>
+    <t>blastoise silver</t>
+  </si>
+  <si>
+    <t>bulbasaur green</t>
+  </si>
+  <si>
+    <t>celebi green</t>
+  </si>
+  <si>
+    <t>chansey green</t>
+  </si>
+  <si>
+    <t>chansey pink</t>
+  </si>
+  <si>
+    <t>chansey silver</t>
+  </si>
+  <si>
+    <t>charizard blue</t>
+  </si>
+  <si>
+    <t>charizard gold</t>
+  </si>
+  <si>
+    <t>charizard red</t>
+  </si>
+  <si>
+    <t>charizard silver</t>
+  </si>
+  <si>
+    <t>chespin silver</t>
+  </si>
+  <si>
+    <t>chikorita green</t>
+  </si>
+  <si>
+    <t>chimchar red</t>
+  </si>
+  <si>
+    <t>corviknight silver</t>
+  </si>
+  <si>
+    <t>crobat pink</t>
+  </si>
+  <si>
+    <t>cyndaquil red</t>
+  </si>
+  <si>
+    <t>darkrai gold</t>
+  </si>
+  <si>
+    <t>darkrai silver</t>
+  </si>
+  <si>
+    <t>darkrai umbreon silver</t>
+  </si>
+  <si>
+    <t>darmanitan blue</t>
+  </si>
+  <si>
+    <t>deoxys espeon silver</t>
+  </si>
+  <si>
+    <t>deoxys red</t>
+  </si>
+  <si>
+    <t>deoxys red 2</t>
+  </si>
+  <si>
+    <t>deoxys silver</t>
+  </si>
+  <si>
+    <t>dialga blue</t>
+  </si>
+  <si>
+    <t>dialga blue 2</t>
+  </si>
+  <si>
+    <t>dialga blue 3</t>
+  </si>
+  <si>
+    <t>dialga silver</t>
+  </si>
+  <si>
+    <t>dragonite gold</t>
+  </si>
+  <si>
+    <t>dragonite gold 2</t>
+  </si>
+  <si>
+    <t>eevee blue</t>
+  </si>
+  <si>
+    <t>eevee blue 2</t>
+  </si>
+  <si>
+    <t>eevee gold</t>
+  </si>
+  <si>
+    <t>eevee gold 2</t>
+  </si>
+  <si>
+    <t>eevee pink</t>
+  </si>
+  <si>
+    <t>eevee red</t>
+  </si>
+  <si>
+    <t>eevee silver</t>
+  </si>
+  <si>
+    <t>empoleon blue</t>
+  </si>
+  <si>
+    <t>energy black</t>
+  </si>
+  <si>
+    <t>energy black 2</t>
+  </si>
+  <si>
+    <t>energy blue</t>
+  </si>
+  <si>
+    <t>energy blue 2</t>
+  </si>
+  <si>
+    <t>energy brown</t>
+  </si>
+  <si>
+    <t>energy brown 2</t>
+  </si>
+  <si>
+    <t>energy gold</t>
+  </si>
+  <si>
+    <t>energy gold 2</t>
+  </si>
+  <si>
+    <t>energy gold 3</t>
+  </si>
+  <si>
+    <t>energy green</t>
+  </si>
+  <si>
+    <t>energy green 2</t>
+  </si>
+  <si>
+    <t>energy pink</t>
+  </si>
+  <si>
+    <t>energy purple</t>
+  </si>
+  <si>
+    <t>energy purple 2</t>
+  </si>
+  <si>
+    <t>energy red</t>
+  </si>
+  <si>
+    <t>energy red2</t>
+  </si>
+  <si>
+    <t>energy silver</t>
+  </si>
+  <si>
+    <t>energy silver 2</t>
+  </si>
+  <si>
+    <t>entei red</t>
+  </si>
+  <si>
+    <t>espeon pink</t>
+  </si>
+  <si>
+    <t>espeon purple</t>
+  </si>
+  <si>
+    <t>fennekin silver</t>
+  </si>
+  <si>
+    <t>flareon red</t>
+  </si>
+  <si>
+    <t>flygon green</t>
+  </si>
+  <si>
+    <t>froakie chespin fennekin silver</t>
+  </si>
+  <si>
+    <t>froakie silver</t>
+  </si>
+  <si>
+    <t>garchomp gold</t>
+  </si>
+  <si>
+    <t>gardevoir purple</t>
+  </si>
+  <si>
+    <t>gardevoir silver</t>
+  </si>
+  <si>
+    <t>gardevoir silver 2</t>
+  </si>
+  <si>
+    <t>genesect purple</t>
+  </si>
+  <si>
+    <t>genesect silver</t>
+  </si>
+  <si>
+    <t>glaceon blue</t>
+  </si>
+  <si>
+    <t>gloom green</t>
+  </si>
+  <si>
+    <t>grookey green</t>
+  </si>
+  <si>
+    <t>groudon red</t>
+  </si>
+  <si>
+    <t>gyarados blue</t>
+  </si>
+  <si>
+    <t>gyarados gold</t>
+  </si>
+  <si>
+    <t>gyarados red</t>
+  </si>
+  <si>
+    <t>hydreigon silver</t>
+  </si>
+  <si>
+    <t>infernape gallade gold</t>
+  </si>
+  <si>
+    <t>jigglypuff pink</t>
+  </si>
+  <si>
+    <t>jirachi gold</t>
+  </si>
+  <si>
+    <t>jolteon silver</t>
+  </si>
+  <si>
+    <t>koraidon red</t>
+  </si>
+  <si>
+    <t>kyogre blue</t>
+  </si>
+  <si>
+    <t>leafeon green</t>
+  </si>
+  <si>
+    <t>litten red</t>
+  </si>
+  <si>
+    <t>lucario gold</t>
+  </si>
+  <si>
+    <t>lucario red</t>
+  </si>
+  <si>
+    <t>lugia silver</t>
+  </si>
+  <si>
+    <t>lunala purple</t>
+  </si>
+  <si>
+    <t>magmortar electrivire gold</t>
+  </si>
+  <si>
+    <t>magmortar electrivire red</t>
+  </si>
+  <si>
+    <t>manaphy blue</t>
+  </si>
+  <si>
+    <t>melmetal silver</t>
+  </si>
+  <si>
+    <t>metagross silver</t>
+  </si>
+  <si>
+    <t>mewtwo purple</t>
+  </si>
+  <si>
+    <t>mewtwo purple 2</t>
+  </si>
+  <si>
+    <t>mew blue</t>
+  </si>
+  <si>
+    <t>mew pink</t>
+  </si>
+  <si>
+    <t>mew pink 2</t>
+  </si>
+  <si>
+    <t>mew silver</t>
+  </si>
+  <si>
+    <t>miraidon purple</t>
+  </si>
+  <si>
+    <t>munchlax gold</t>
+  </si>
+  <si>
+    <t>munchlax silver</t>
+  </si>
+  <si>
+    <t>ninetales red</t>
+  </si>
+  <si>
+    <t>ninetales silver</t>
+  </si>
+  <si>
+    <t>onix brown</t>
+  </si>
+  <si>
+    <t>palkia pink 1</t>
+  </si>
+  <si>
+    <t>palkia pink 2</t>
+  </si>
+  <si>
+    <t>palkia pink 3</t>
+  </si>
+  <si>
+    <t>palkia silver</t>
+  </si>
+  <si>
+    <t>pichu gold</t>
+  </si>
+  <si>
+    <t>pikachu charizard mewtwo silver</t>
+  </si>
+  <si>
+    <t>pikachu gold</t>
+  </si>
+  <si>
+    <t>pikachu gold 1</t>
+  </si>
+  <si>
+    <t>pikachu gold 2</t>
+  </si>
+  <si>
+    <t>pikachu gold 3</t>
+  </si>
+  <si>
+    <t>pikachu red 1</t>
+  </si>
+  <si>
+    <t>pikachu silver 1</t>
+  </si>
+  <si>
+    <t>pikachu silver 2</t>
+  </si>
+  <si>
+    <t>piplup blue</t>
+  </si>
+  <si>
+    <t>plasma blue</t>
+  </si>
+  <si>
+    <t>plasma silver</t>
+  </si>
+  <si>
+    <t>pokeball red</t>
+  </si>
+  <si>
+    <t>popplio blue</t>
+  </si>
+  <si>
+    <t>primal groudon red</t>
+  </si>
+  <si>
+    <t>primal kyogre blue</t>
+  </si>
+  <si>
+    <t>raichu gold</t>
+  </si>
+  <si>
+    <t>raichu gold 2</t>
+  </si>
+  <si>
+    <t>raikou gold</t>
+  </si>
+  <si>
+    <t>rayquaza gold</t>
+  </si>
+  <si>
+    <t>rayquaza green</t>
+  </si>
+  <si>
+    <t>rayquaza silver</t>
+  </si>
+  <si>
+    <t>reshiram zekrom silver</t>
+  </si>
+  <si>
+    <t>rocket silver</t>
+  </si>
+  <si>
+    <t>rowlett green</t>
+  </si>
+  <si>
+    <t>salamance gold</t>
+  </si>
+  <si>
+    <t>sceptile green</t>
+  </si>
+  <si>
+    <t>scorbunny red</t>
+  </si>
+  <si>
+    <t>sirfetchd green</t>
+  </si>
+  <si>
+    <t>slowpoke pink</t>
+  </si>
+  <si>
+    <t>snom blue</t>
+  </si>
+  <si>
+    <t>sobble blue</t>
+  </si>
+  <si>
+    <t>solgaleo gold</t>
+  </si>
+  <si>
+    <t>sprigatito silver</t>
+  </si>
+  <si>
+    <t>steelix silver</t>
+  </si>
+  <si>
+    <t>suicune silver</t>
+  </si>
+  <si>
+    <t>swampert blue</t>
+  </si>
+  <si>
+    <t>sylveon pink</t>
+  </si>
+  <si>
+    <t>terapagos blue</t>
+  </si>
+  <si>
+    <t>togepi cleffa igglybuff pink</t>
+  </si>
+  <si>
+    <t>totodile blue</t>
+  </si>
+  <si>
+    <t>treeko torchic mudkip silver</t>
+  </si>
+  <si>
+    <t>turtwig green</t>
+  </si>
+  <si>
+    <t>tyranitar blue</t>
+  </si>
+  <si>
+    <t>tyranitar gold</t>
+  </si>
+  <si>
+    <t>tyranitar silver</t>
+  </si>
+  <si>
+    <t>umbreon black</t>
+  </si>
+  <si>
+    <t>umbreon pink</t>
+  </si>
+  <si>
+    <t>urshifu blue</t>
+  </si>
+  <si>
+    <t>urshifu red</t>
+  </si>
+  <si>
+    <t>vaporeon silver</t>
+  </si>
+  <si>
+    <t>venusaur green</t>
+  </si>
+  <si>
+    <t>volcanion red</t>
+  </si>
+  <si>
+    <t>wooloo silver</t>
+  </si>
+  <si>
+    <t>xerneas blue</t>
+  </si>
+  <si>
+    <t>xerneas silver</t>
+  </si>
+  <si>
+    <t>yampa gold</t>
+  </si>
+  <si>
+    <t>yveltal red</t>
+  </si>
+  <si>
+    <t>yveltal silver</t>
+  </si>
+  <si>
+    <t>zapdos gold</t>
+  </si>
+  <si>
+    <t>zoroark silver</t>
+  </si>
+  <si>
+    <t>Hiker Ben</t>
+  </si>
+  <si>
+    <t>Evening 3</t>
+  </si>
+  <si>
+    <t>Bad Dude Wayne</t>
+  </si>
+  <si>
+    <t>Night 3</t>
+  </si>
+  <si>
+    <t>rocket blue</t>
+  </si>
+  <si>
+    <t>rocket red</t>
+  </si>
+  <si>
+    <t>Rocket Grunt Damien</t>
+  </si>
+  <si>
+    <t>Rocket Grunt Penny</t>
   </si>
 </sst>
 </file>
@@ -791,13 +1364,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CABA093D-E10D-4AFA-84B7-B1B7EB5F6B16}" name="Table1" displayName="Table1" ref="A1:C179" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:C179" xr:uid="{CABA093D-E10D-4AFA-84B7-B1B7EB5F6B16}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C177">
-    <sortCondition ref="B1:B179"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CABA093D-E10D-4AFA-84B7-B1B7EB5F6B16}" name="Table1" displayName="Table1" ref="A1:D181" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D181" xr:uid="{CABA093D-E10D-4AFA-84B7-B1B7EB5F6B16}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:D179">
+    <sortCondition ref="C1:C181"/>
   </sortState>
-  <tableColumns count="3">
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{B1B3F4BF-11CF-4DCD-BBFF-800CA95AB652}" name="Coin"/>
+    <tableColumn id="4" xr3:uid="{F48141CC-50B0-4B5B-B36E-7B26E2763CED}" name="Coin Name"/>
     <tableColumn id="2" xr3:uid="{2B45EC9D-2894-4946-81C0-66214EF570D9}" name="granted by name"/>
     <tableColumn id="3" xr3:uid="{7746DE0B-7B46-4C19-BAE4-2167203617DB}" name="granted day"/>
   </tableColumns>
@@ -1122,1186 +1696,1779 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E36B1B59-0D5E-4C8D-AEE2-CA809DBB4E7C}">
-  <dimension ref="A1:C179"/>
+  <dimension ref="A1:D181"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="1" max="1" width="40.7109375" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="40.7109375" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>181</v>
+        <v>230</v>
       </c>
       <c r="C3" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>231</v>
+      </c>
+      <c r="C4" t="s">
+        <v>205</v>
+      </c>
+      <c r="D4" t="s">
         <v>206</v>
       </c>
-      <c r="C4" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>235</v>
+      </c>
+      <c r="C8" t="s">
+        <v>223</v>
+      </c>
+      <c r="D8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>236</v>
+      </c>
+      <c r="C9" t="s">
+        <v>181</v>
+      </c>
+      <c r="D9" t="s">
         <v>182</v>
       </c>
-      <c r="C9" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
       <c r="C11" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+      <c r="D11" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="C12" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="D12" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
       <c r="B13" t="s">
+        <v>240</v>
+      </c>
+      <c r="C13" t="s">
+        <v>183</v>
+      </c>
+      <c r="D13" t="s">
         <v>184</v>
       </c>
-      <c r="C13" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>219</v>
+        <v>248</v>
       </c>
       <c r="C21" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+      <c r="D21" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>252</v>
+      </c>
+      <c r="C25" t="s">
+        <v>409</v>
+      </c>
+      <c r="D25" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+        <v>263</v>
+      </c>
+      <c r="C36" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>186</v>
+        <v>271</v>
       </c>
       <c r="C44" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+      <c r="D44" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>192</v>
+        <v>275</v>
       </c>
       <c r="C48" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+      <c r="D48" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>193</v>
+        <v>276</v>
       </c>
       <c r="C49" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+      <c r="D49" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>194</v>
+        <v>277</v>
       </c>
       <c r="C50" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+      <c r="D50" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>195</v>
+        <v>278</v>
       </c>
       <c r="C51" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+        <v>194</v>
+      </c>
+      <c r="D51" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>188</v>
+        <v>279</v>
       </c>
       <c r="C52" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+      <c r="D52" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>197</v>
+        <v>282</v>
       </c>
       <c r="C55" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+        <v>196</v>
+      </c>
+      <c r="D55" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>54</v>
       </c>
-      <c r="C56" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>198</v>
+        <v>285</v>
       </c>
       <c r="C58" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+      <c r="D58" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>199</v>
+        <v>287</v>
       </c>
       <c r="C60" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+      <c r="D60" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>187</v>
+        <v>290</v>
       </c>
       <c r="C63" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+      <c r="D63" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B70" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B71" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B72" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B73" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>73</v>
       </c>
       <c r="B75" t="s">
+        <v>302</v>
+      </c>
+      <c r="C75" t="s">
+        <v>205</v>
+      </c>
+      <c r="D75" t="s">
         <v>206</v>
       </c>
-      <c r="C75" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>74</v>
       </c>
       <c r="B76" t="s">
-        <v>213</v>
+        <v>303</v>
       </c>
       <c r="C76" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+      <c r="D76" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B77" t="s">
+        <v>304</v>
+      </c>
+      <c r="C77" t="s">
+        <v>225</v>
+      </c>
+      <c r="D77" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B78" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B81" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>189</v>
+        <v>309</v>
       </c>
       <c r="C82" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+      <c r="D82" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>213</v>
+      </c>
+      <c r="B83" t="s">
+        <v>310</v>
+      </c>
+      <c r="C83" t="s">
         <v>214</v>
       </c>
-      <c r="B83" t="s">
-        <v>215</v>
-      </c>
-      <c r="C83" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D83" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>81</v>
       </c>
       <c r="B84" t="s">
-        <v>190</v>
+        <v>311</v>
       </c>
       <c r="C84" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+      <c r="D84" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>82</v>
       </c>
       <c r="B85" t="s">
+        <v>312</v>
+      </c>
+      <c r="C85" t="s">
+        <v>205</v>
+      </c>
+      <c r="D85" t="s">
         <v>206</v>
       </c>
-      <c r="C85" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>84</v>
       </c>
       <c r="B87" t="s">
-        <v>217</v>
+        <v>314</v>
       </c>
       <c r="C87" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+        <v>216</v>
+      </c>
+      <c r="D87" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B88" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B89" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B90" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>88</v>
       </c>
       <c r="B91" t="s">
-        <v>212</v>
+        <v>318</v>
       </c>
       <c r="C91" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+      <c r="D91" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B92" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B93" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B94" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B95" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>93</v>
       </c>
       <c r="B96" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+        <v>323</v>
+      </c>
+      <c r="C96" t="s">
+        <v>210</v>
+      </c>
+      <c r="D96" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B97" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B98" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B99" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B100" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B101" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B102" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B103" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B104" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B105" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>103</v>
       </c>
       <c r="B106" t="s">
-        <v>200</v>
+        <v>333</v>
       </c>
       <c r="C106" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+      <c r="D106" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B107" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>105</v>
       </c>
-      <c r="C108" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B108" t="s">
+        <v>335</v>
+      </c>
+      <c r="D108" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B109" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>107</v>
       </c>
       <c r="B110" t="s">
+        <v>337</v>
+      </c>
+      <c r="C110" t="s">
+        <v>207</v>
+      </c>
+      <c r="D110" t="s">
         <v>208</v>
       </c>
-      <c r="C110" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>108</v>
       </c>
       <c r="B111" t="s">
+        <v>338</v>
+      </c>
+      <c r="C111" t="s">
+        <v>207</v>
+      </c>
+      <c r="D111" t="s">
         <v>208</v>
       </c>
-      <c r="C111" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B112" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B113" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B114" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B115" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B116" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B117" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B118" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B119" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>117</v>
       </c>
       <c r="B120" t="s">
+        <v>347</v>
+      </c>
+      <c r="C120" t="s">
+        <v>205</v>
+      </c>
+      <c r="D120" t="s">
         <v>206</v>
       </c>
-      <c r="C120" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B121" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B123" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>121</v>
       </c>
       <c r="B124" t="s">
-        <v>191</v>
+        <v>351</v>
       </c>
       <c r="C124" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+      <c r="D124" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>123</v>
       </c>
       <c r="B126" t="s">
-        <v>201</v>
+        <v>353</v>
       </c>
       <c r="C126" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+      <c r="D126" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B127" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B128" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B129" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B130" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B131" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B132" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B133" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B134" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B135" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B136" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B137" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B138" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B139" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B140" t="s">
+        <v>367</v>
+      </c>
+      <c r="C140" t="s">
+        <v>226</v>
+      </c>
+      <c r="D140" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>138</v>
       </c>
       <c r="B141" t="s">
-        <v>205</v>
+        <v>368</v>
       </c>
       <c r="C141" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
+      <c r="D141" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B142" t="s">
+        <v>411</v>
+      </c>
+      <c r="C142" t="s">
+        <v>413</v>
+      </c>
+      <c r="D142" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B143" t="s">
+        <v>412</v>
+      </c>
+      <c r="C143" t="s">
+        <v>414</v>
+      </c>
+      <c r="D143" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
+      <c r="B144" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A144" t="s">
+      <c r="B145" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
+      <c r="B146" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A146" t="s">
+      <c r="B147" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
         <v>143</v>
       </c>
-      <c r="B146" t="s">
+      <c r="B148" t="s">
+        <v>373</v>
+      </c>
+      <c r="C148" t="s">
+        <v>202</v>
+      </c>
+      <c r="D148" t="s">
         <v>203</v>
       </c>
-      <c r="C146" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A147" t="s">
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
+      <c r="B149" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
+      <c r="B150" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
+      <c r="B151" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
+      <c r="B152" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
         <v>148</v>
       </c>
-      <c r="B151" t="s">
-        <v>220</v>
-      </c>
-      <c r="C151" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
+      <c r="B153" t="s">
+        <v>378</v>
+      </c>
+      <c r="C153" t="s">
+        <v>219</v>
+      </c>
+      <c r="D153" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
+      <c r="B154" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A154" t="s">
+      <c r="B155" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A155" t="s">
+      <c r="B156" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A156" t="s">
+      <c r="B157" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A157" t="s">
+      <c r="B158" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
         <v>154</v>
       </c>
-      <c r="B157" t="s">
+      <c r="B159" t="s">
+        <v>384</v>
+      </c>
+      <c r="C159" t="s">
+        <v>205</v>
+      </c>
+      <c r="D159" t="s">
         <v>206</v>
       </c>
-      <c r="C157" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A158" t="s">
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A159" t="s">
+      <c r="B160" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A160" t="s">
+      <c r="B161" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A161" t="s">
+      <c r="B162" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
         <v>158</v>
       </c>
-      <c r="B161" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A162" t="s">
+      <c r="B163" t="s">
+        <v>388</v>
+      </c>
+      <c r="C163" t="s">
+        <v>195</v>
+      </c>
+      <c r="D163" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A163" t="s">
+      <c r="B164" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>227</v>
+      </c>
+      <c r="B165" t="s">
+        <v>390</v>
+      </c>
+      <c r="C165" t="s">
+        <v>407</v>
+      </c>
+      <c r="D165" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A164" t="s">
+      <c r="B166" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A165" t="s">
+      <c r="B167" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A166" t="s">
+      <c r="B168" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A167" t="s">
+      <c r="B169" t="s">
+        <v>394</v>
+      </c>
+      <c r="C169" t="s">
+        <v>205</v>
+      </c>
+      <c r="D169" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
         <v>164</v>
       </c>
-      <c r="B167" t="s">
+      <c r="B170" t="s">
+        <v>395</v>
+      </c>
+      <c r="C170" t="s">
+        <v>205</v>
+      </c>
+      <c r="D170" t="s">
         <v>206</v>
       </c>
-      <c r="C167" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A168" t="s">
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
         <v>165</v>
       </c>
-      <c r="B168" t="s">
+      <c r="B171" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>166</v>
+      </c>
+      <c r="B172" t="s">
+        <v>397</v>
+      </c>
+      <c r="C172" t="s">
+        <v>222</v>
+      </c>
+      <c r="D172" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>167</v>
+      </c>
+      <c r="B173" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>168</v>
+      </c>
+      <c r="B174" t="s">
+        <v>399</v>
+      </c>
+      <c r="C174" t="s">
+        <v>205</v>
+      </c>
+      <c r="D174" t="s">
         <v>206</v>
       </c>
-      <c r="C168" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A169" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A170" t="s">
-        <v>167</v>
-      </c>
-      <c r="B170" t="s">
-        <v>223</v>
-      </c>
-      <c r="C170" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A171" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A172" t="s">
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
         <v>169</v>
       </c>
-      <c r="B172" t="s">
+      <c r="B175" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>170</v>
+      </c>
+      <c r="B176" t="s">
+        <v>401</v>
+      </c>
+      <c r="C176" t="s">
+        <v>205</v>
+      </c>
+      <c r="D176" t="s">
         <v>206</v>
       </c>
-      <c r="C172" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A173" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A174" t="s">
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
         <v>171</v>
       </c>
-      <c r="B174" t="s">
+      <c r="B177" t="s">
+        <v>402</v>
+      </c>
+      <c r="C177" t="s">
+        <v>201</v>
+      </c>
+      <c r="D177" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>172</v>
+      </c>
+      <c r="B178" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>173</v>
+      </c>
+      <c r="B179" t="s">
+        <v>404</v>
+      </c>
+      <c r="C179" t="s">
+        <v>205</v>
+      </c>
+      <c r="D179" t="s">
         <v>206</v>
       </c>
-      <c r="C174" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A175" t="s">
-        <v>172</v>
-      </c>
-      <c r="B175" t="s">
-        <v>202</v>
-      </c>
-      <c r="C175" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A176" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A177" t="s">
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
         <v>174</v>
       </c>
-      <c r="B177" t="s">
-        <v>206</v>
-      </c>
-      <c r="C177" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A178" t="s">
+      <c r="B180" t="s">
+        <v>405</v>
+      </c>
+      <c r="C180" t="s">
+        <v>217</v>
+      </c>
+      <c r="D180" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
         <v>175</v>
       </c>
-      <c r="B178" t="s">
-        <v>218</v>
-      </c>
-      <c r="C178" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A179" t="s">
-        <v>176</v>
+      <c r="B181" t="s">
+        <v>406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Koga night 3 npc and updated coin tracker to be fully up to date
</commit_message>
<xml_diff>
--- a/Coin_tracker.xlsx
+++ b/Coin_tracker.xlsx
@@ -2,1285 +2,1284 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD2F134-986D-4142-84C3-B6881BF76845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34EF1D5-10FB-4372-A8A7-65986C101030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{2902C7A9-D4C7-4F9F-B9D2-2E43E3BE476A}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="420">
+  <si>
+    <t>Coin</t>
+  </si>
+  <si>
+    <t>Coin Name</t>
+  </si>
+  <si>
+    <t>granted by name</t>
+  </si>
+  <si>
+    <t>granted day</t>
+  </si>
   <si>
     <t>coin_alakazam_purple.png</t>
   </si>
   <si>
+    <t>alakazam purple</t>
+  </si>
+  <si>
     <t>coin_arcanine_red.png</t>
   </si>
   <si>
+    <t>arcanine red</t>
+  </si>
+  <si>
+    <t>FIREBREATHER KENNETH</t>
+  </si>
+  <si>
+    <t>Evening 2</t>
+  </si>
+  <si>
     <t>coin_arceus_silver.png</t>
   </si>
   <si>
+    <t>arceus silver</t>
+  </si>
+  <si>
+    <t>COIN SHOP</t>
+  </si>
+  <si>
+    <t>Day 3+</t>
+  </si>
+  <si>
     <t>coin_back_basic.png</t>
   </si>
   <si>
+    <t>back basic</t>
+  </si>
+  <si>
     <t>coin_blastoise_blue.png</t>
   </si>
   <si>
+    <t>blastoise blue</t>
+  </si>
+  <si>
     <t>coin_blastoise_blue_2.png</t>
   </si>
   <si>
+    <t>blastoise blue 2</t>
+  </si>
+  <si>
     <t>coin_blastoise_silver.png</t>
   </si>
   <si>
+    <t>blastoise silver</t>
+  </si>
+  <si>
+    <t>CARD ELDER RAYNE</t>
+  </si>
+  <si>
+    <t>Evening 3</t>
+  </si>
+  <si>
     <t>coin_bulbasaur_green.png</t>
   </si>
   <si>
+    <t>bulbasaur green</t>
+  </si>
+  <si>
+    <t>GARDENER CALLUM</t>
+  </si>
+  <si>
+    <t>Evening 1</t>
+  </si>
+  <si>
     <t>coin_celebi_green.png</t>
   </si>
   <si>
+    <t>celebi green</t>
+  </si>
+  <si>
     <t>coin_chansey_green.png</t>
   </si>
   <si>
+    <t>chansey green</t>
+  </si>
+  <si>
+    <t>YOUNG TWIN ANNA</t>
+  </si>
+  <si>
+    <t>Day 3</t>
+  </si>
+  <si>
     <t>coin_chansey_pink.png</t>
   </si>
   <si>
+    <t>chansey pink</t>
+  </si>
+  <si>
+    <t>YOUNG TWIN NELLA</t>
+  </si>
+  <si>
     <t>coin_chansey_silver.png</t>
   </si>
   <si>
+    <t>chansey silver</t>
+  </si>
+  <si>
+    <t>SCHOOLBOY ADAM</t>
+  </si>
+  <si>
+    <t>Day 1</t>
+  </si>
+  <si>
     <t>coin_charizard_blue.png</t>
   </si>
   <si>
+    <t>charizard blue</t>
+  </si>
+  <si>
     <t>coin_charizard_gold.png</t>
   </si>
   <si>
+    <t>charizard gold</t>
+  </si>
+  <si>
     <t>coin_charizard_red.png</t>
   </si>
   <si>
+    <t>charizard red</t>
+  </si>
+  <si>
     <t>coin_charizard_silver.png</t>
   </si>
   <si>
+    <t>charizard silver</t>
+  </si>
+  <si>
     <t>coin_chespin_silver.png</t>
   </si>
   <si>
+    <t>chespin silver</t>
+  </si>
+  <si>
     <t>coin_chikorita_green.png</t>
   </si>
   <si>
+    <t>chikorita green</t>
+  </si>
+  <si>
     <t>coin_chimchar_red.png</t>
   </si>
   <si>
+    <t>chimchar red</t>
+  </si>
+  <si>
     <t>coin_corviknight_silver.png</t>
   </si>
   <si>
+    <t>corviknight silver</t>
+  </si>
+  <si>
+    <t>BIRDSPOTTER TAMSIN</t>
+  </si>
+  <si>
+    <t>Day 2</t>
+  </si>
+  <si>
     <t>coin_crobat_pink.png</t>
   </si>
   <si>
+    <t>crobat pink</t>
+  </si>
+  <si>
     <t>coin_cyndaquil_red.png</t>
   </si>
   <si>
+    <t>cyndaquil red</t>
+  </si>
+  <si>
     <t>coin_darkrai_gold.png</t>
   </si>
   <si>
+    <t>darkrai gold</t>
+  </si>
+  <si>
     <t>coin_darkrai_silver.png</t>
   </si>
   <si>
+    <t>darkrai silver</t>
+  </si>
+  <si>
+    <t>SUNBATHING DUDE 1 NIGHT</t>
+  </si>
+  <si>
+    <t>Night 2</t>
+  </si>
+  <si>
     <t>coin_darkrai_umbreon_silver.png</t>
   </si>
   <si>
+    <t>darkrai umbreon silver</t>
+  </si>
+  <si>
     <t>coin_darmanitan_blue.png</t>
   </si>
   <si>
+    <t>darmanitan blue</t>
+  </si>
+  <si>
     <t>coin_deoxys_espeon_silver.png</t>
   </si>
   <si>
+    <t>deoxys espeon silver</t>
+  </si>
+  <si>
     <t>coin_deoxys_red.png</t>
   </si>
   <si>
+    <t>deoxys red</t>
+  </si>
+  <si>
     <t>coin_deoxys_red_2.png</t>
   </si>
   <si>
+    <t>deoxys red 2</t>
+  </si>
+  <si>
     <t>coin_deoxys_silver.png</t>
   </si>
   <si>
+    <t>deoxys silver</t>
+  </si>
+  <si>
     <t>coin_dialga_blue.png</t>
   </si>
   <si>
+    <t>dialga blue</t>
+  </si>
+  <si>
     <t>coin_dialga_blue_2.png</t>
   </si>
   <si>
+    <t>dialga blue 2</t>
+  </si>
+  <si>
     <t>coin_dialga_blue_3.png</t>
   </si>
   <si>
+    <t>dialga blue 3</t>
+  </si>
+  <si>
     <t>coin_dialga_silver.png</t>
   </si>
   <si>
+    <t>dialga silver</t>
+  </si>
+  <si>
     <t>coin_dragonite_gold.png</t>
   </si>
   <si>
+    <t>dragonite gold</t>
+  </si>
+  <si>
+    <t>SS ANNE TOURIST EDMUND</t>
+  </si>
+  <si>
     <t>coin_dragonite_gold_2.png</t>
   </si>
   <si>
+    <t>dragonite gold 2</t>
+  </si>
+  <si>
     <t>coin_eevee_blue.png</t>
   </si>
   <si>
+    <t>eevee blue</t>
+  </si>
+  <si>
     <t>coin_eevee_blue_2.png</t>
   </si>
   <si>
+    <t>eevee blue 2</t>
+  </si>
+  <si>
     <t>coin_eevee_gold.png</t>
   </si>
   <si>
+    <t>eevee gold</t>
+  </si>
+  <si>
     <t>coin_eevee_gold_2.png</t>
   </si>
   <si>
+    <t>eevee gold 2</t>
+  </si>
+  <si>
     <t>coin_eevee_pink.png</t>
   </si>
   <si>
+    <t>eevee pink</t>
+  </si>
+  <si>
     <t>coin_eevee_red.png</t>
   </si>
   <si>
+    <t>eevee red</t>
+  </si>
+  <si>
     <t>coin_eevee_silver.png</t>
   </si>
   <si>
+    <t>eevee silver</t>
+  </si>
+  <si>
+    <t>PAINTER JERICHO</t>
+  </si>
+  <si>
     <t>coin_empoleon_blue.png</t>
   </si>
   <si>
+    <t>empoleon blue</t>
+  </si>
+  <si>
     <t>coin_energy_black.png</t>
   </si>
   <si>
+    <t>energy black</t>
+  </si>
+  <si>
     <t>coin_energy_black_2.png</t>
   </si>
   <si>
+    <t>energy black 2</t>
+  </si>
+  <si>
     <t>coin_energy_blue.png</t>
   </si>
   <si>
+    <t>energy blue</t>
+  </si>
+  <si>
+    <t>SWIMMER JORDAN</t>
+  </si>
+  <si>
     <t>coin_energy_blue_2.png</t>
   </si>
   <si>
+    <t>energy blue 2</t>
+  </si>
+  <si>
+    <t>SWIMMER TODD</t>
+  </si>
+  <si>
     <t>coin_energy_brown.png</t>
   </si>
   <si>
+    <t>energy brown</t>
+  </si>
+  <si>
+    <t>BATTLEGIRL SOFIA</t>
+  </si>
+  <si>
     <t>coin_energy_brown_2.png</t>
   </si>
   <si>
+    <t>energy brown 2</t>
+  </si>
+  <si>
+    <t>SAILOR BOB</t>
+  </si>
+  <si>
     <t>coin_energy_gold.png</t>
   </si>
   <si>
+    <t>energy gold</t>
+  </si>
+  <si>
+    <t>ENGINEER ALLAN</t>
+  </si>
+  <si>
     <t>coin_energy_gold_2.png</t>
   </si>
   <si>
+    <t>energy gold 2</t>
+  </si>
+  <si>
     <t>coin_energy_gold_3.png</t>
   </si>
   <si>
+    <t>energy gold 3</t>
+  </si>
+  <si>
     <t>coin_energy_green.png</t>
   </si>
   <si>
+    <t>energy green</t>
+  </si>
+  <si>
+    <t>BUG CATCHER ALEX</t>
+  </si>
+  <si>
     <t>coin_energy_green_2.png</t>
   </si>
   <si>
+    <t>energy green 2</t>
+  </si>
+  <si>
+    <t>BUG CATCHER JOHNNY</t>
+  </si>
+  <si>
     <t>coin_energy_pink.png</t>
   </si>
   <si>
+    <t>energy pink</t>
+  </si>
+  <si>
     <t>coin_energy_purple.png</t>
   </si>
   <si>
+    <t>energy purple</t>
+  </si>
+  <si>
+    <t>PSYCHIC BRIENNE</t>
+  </si>
+  <si>
     <t>coin_energy_purple_2.png</t>
   </si>
   <si>
+    <t>energy purple 2</t>
+  </si>
+  <si>
     <t>coin_energy_red.png</t>
   </si>
   <si>
+    <t>energy red</t>
+  </si>
+  <si>
+    <t>FIREBREATHER DARRYL</t>
+  </si>
+  <si>
     <t>coin_energy_red2.png</t>
   </si>
   <si>
+    <t>energy red2</t>
+  </si>
+  <si>
     <t>coin_energy_silver.png</t>
   </si>
   <si>
+    <t>energy silver</t>
+  </si>
+  <si>
     <t>coin_energy_silver_2.png</t>
   </si>
   <si>
+    <t>energy silver 2</t>
+  </si>
+  <si>
+    <t>YOUNGSTER JOEY</t>
+  </si>
+  <si>
     <t>coin_entei_red.png</t>
   </si>
   <si>
+    <t>entei red</t>
+  </si>
+  <si>
     <t>coin_espeon_pink.png</t>
   </si>
   <si>
+    <t>espeon pink</t>
+  </si>
+  <si>
     <t>coin_espeon_purple.png</t>
   </si>
   <si>
+    <t>espeon purple</t>
+  </si>
+  <si>
     <t>coin_fennekin_silver.png</t>
   </si>
   <si>
+    <t>fennekin silver</t>
+  </si>
+  <si>
     <t>coin_flareon_red.png</t>
   </si>
   <si>
+    <t>flareon red</t>
+  </si>
+  <si>
     <t>coin_flygon_green.png</t>
   </si>
   <si>
+    <t>flygon green</t>
+  </si>
+  <si>
     <t>coin_froakie_chespin_fennekin_silver.png</t>
   </si>
   <si>
+    <t>froakie chespin fennekin silver</t>
+  </si>
+  <si>
     <t>coin_froakie_silver.png</t>
   </si>
   <si>
+    <t>froakie silver</t>
+  </si>
+  <si>
     <t>coin_garchomp_gold.png</t>
   </si>
   <si>
+    <t>garchomp gold</t>
+  </si>
+  <si>
     <t>coin_gardevoir_purple.png</t>
   </si>
   <si>
+    <t>gardevoir purple</t>
+  </si>
+  <si>
     <t>coin_gardevoir_silver.png</t>
   </si>
   <si>
+    <t>gardevoir silver</t>
+  </si>
+  <si>
     <t>coin_gardevoir_silver_2.png</t>
   </si>
   <si>
+    <t>gardevoir silver 2</t>
+  </si>
+  <si>
     <t>coin_genesect_purple.png</t>
   </si>
   <si>
+    <t>genesect purple</t>
+  </si>
+  <si>
+    <t>BUG CATCHER FRANKIE</t>
+  </si>
+  <si>
     <t>coin_genesect_silver.png</t>
   </si>
   <si>
+    <t>genesect silver</t>
+  </si>
+  <si>
+    <t>CARD ELDER WAVERLY</t>
+  </si>
+  <si>
     <t>coin_glaceon_blue.png</t>
   </si>
   <si>
+    <t>glaceon blue</t>
+  </si>
+  <si>
     <t>coin_gloom_green.png</t>
   </si>
   <si>
+    <t>gloom green</t>
+  </si>
+  <si>
     <t>coin_grookey_green.png</t>
   </si>
   <si>
+    <t>grookey green</t>
+  </si>
+  <si>
     <t>coin_groudon_red.png</t>
   </si>
   <si>
+    <t>groudon red</t>
+  </si>
+  <si>
     <t>coin_gyarados_blue.png</t>
   </si>
   <si>
+    <t>gyarados blue</t>
+  </si>
+  <si>
+    <t>FISHERMAN DAVE</t>
+  </si>
+  <si>
+    <t>coin_gyarados_gold.png</t>
+  </si>
+  <si>
+    <t>gyarados gold</t>
+  </si>
+  <si>
+    <t>FISHERMAN GARY</t>
+  </si>
+  <si>
     <t>coin_gyarados_red.png</t>
   </si>
   <si>
+    <t>gyarados red</t>
+  </si>
+  <si>
+    <t>FISHERMAN JOHN</t>
+  </si>
+  <si>
     <t>coin_hydreigon_silver.png</t>
   </si>
   <si>
+    <t>hydreigon silver</t>
+  </si>
+  <si>
     <t>coin_infernape_gallade_gold.png</t>
   </si>
   <si>
+    <t>infernape gallade gold</t>
+  </si>
+  <si>
     <t>coin_jigglypuff_pink.png</t>
   </si>
   <si>
+    <t>jigglypuff pink</t>
+  </si>
+  <si>
+    <t>SS ANNE TOURIST ALISSA</t>
+  </si>
+  <si>
     <t>coin_jirachi_gold.png</t>
   </si>
   <si>
+    <t>jirachi gold</t>
+  </si>
+  <si>
     <t>coin_jolteon_silver.png</t>
   </si>
   <si>
+    <t>jolteon silver</t>
+  </si>
+  <si>
     <t>coin_koraidon_red.png</t>
   </si>
   <si>
+    <t>koraidon red</t>
+  </si>
+  <si>
+    <t>ENGINEER BRAD</t>
+  </si>
+  <si>
+    <t>Night 3</t>
+  </si>
+  <si>
     <t>coin_kyogre_blue.png</t>
   </si>
   <si>
+    <t>kyogre blue</t>
+  </si>
+  <si>
+    <t>SWIMMER MELISSA</t>
+  </si>
+  <si>
     <t>coin_leafeon_green.png</t>
   </si>
   <si>
+    <t>leafeon green</t>
+  </si>
+  <si>
     <t>coin_litten_red.png</t>
   </si>
   <si>
+    <t>litten red</t>
+  </si>
+  <si>
     <t>coin_lucario_gold.png</t>
   </si>
   <si>
+    <t>lucario gold</t>
+  </si>
+  <si>
     <t>coin_lucario_red.png</t>
   </si>
   <si>
+    <t>lucario red</t>
+  </si>
+  <si>
     <t>coin_lugia_silver.png</t>
   </si>
   <si>
+    <t>lugia silver</t>
+  </si>
+  <si>
+    <t>BIRDSPOTTER GREGG</t>
+  </si>
+  <si>
     <t>coin_lunala_purple.png</t>
   </si>
   <si>
+    <t>lunala purple</t>
+  </si>
+  <si>
     <t>coin_magmortar_electrivire_gold.png</t>
   </si>
   <si>
+    <t>magmortar electrivire gold</t>
+  </si>
+  <si>
     <t>coin_magmortar_electrivire_red.png</t>
   </si>
   <si>
+    <t>magmortar electrivire red</t>
+  </si>
+  <si>
     <t>coin_manaphy_blue.png</t>
   </si>
   <si>
+    <t>manaphy blue</t>
+  </si>
+  <si>
     <t>coin_melmetal_silver.png</t>
   </si>
   <si>
+    <t>melmetal silver</t>
+  </si>
+  <si>
     <t>coin_metagross_silver.png</t>
   </si>
   <si>
+    <t>metagross silver</t>
+  </si>
+  <si>
     <t>coin_mewtwo_purple.png</t>
   </si>
   <si>
+    <t>mewtwo purple</t>
+  </si>
+  <si>
     <t>coin_mewtwo_purple_2.png</t>
   </si>
   <si>
+    <t>mewtwo purple 2</t>
+  </si>
+  <si>
     <t>coin_mew_blue.png</t>
   </si>
   <si>
+    <t>mew blue</t>
+  </si>
+  <si>
     <t>coin_mew_pink.png</t>
   </si>
   <si>
+    <t>mew pink</t>
+  </si>
+  <si>
+    <t>BEACH KID EVIE</t>
+  </si>
+  <si>
     <t>coin_mew_pink_2.png</t>
   </si>
   <si>
+    <t>mew pink 2</t>
+  </si>
+  <si>
     <t>coin_mew_silver.png</t>
   </si>
   <si>
+    <t>mew silver</t>
+  </si>
+  <si>
     <t>coin_miraidon_purple.png</t>
   </si>
   <si>
+    <t>miraidon purple</t>
+  </si>
+  <si>
     <t>coin_munchlax_gold.png</t>
   </si>
   <si>
+    <t>munchlax gold</t>
+  </si>
+  <si>
+    <t>JUICE BAR</t>
+  </si>
+  <si>
+    <t>Day 2+</t>
+  </si>
+  <si>
     <t>coin_munchlax_silver.png</t>
   </si>
   <si>
+    <t>munchlax silver</t>
+  </si>
+  <si>
     <t>coin_ninetales_red.png</t>
   </si>
   <si>
+    <t>ninetales red</t>
+  </si>
+  <si>
     <t>coin_ninetales_silver.png</t>
   </si>
   <si>
+    <t>ninetales silver</t>
+  </si>
+  <si>
     <t>coin_onix_brown.png</t>
   </si>
   <si>
+    <t>onix brown</t>
+  </si>
+  <si>
+    <t>HIKER MATTHEW</t>
+  </si>
+  <si>
     <t>coin_palkia_pink_1.png</t>
   </si>
   <si>
+    <t>palkia pink 1</t>
+  </si>
+  <si>
     <t>coin_palkia_pink_2.png</t>
   </si>
   <si>
+    <t>palkia pink 2</t>
+  </si>
+  <si>
     <t>coin_palkia_pink_3.png</t>
   </si>
   <si>
+    <t>palkia pink 3</t>
+  </si>
+  <si>
     <t>coin_palkia_silver.png</t>
   </si>
   <si>
+    <t>palkia silver</t>
+  </si>
+  <si>
     <t>coin_pichu_gold.png</t>
   </si>
   <si>
+    <t>pichu gold</t>
+  </si>
+  <si>
     <t>coin_pikachu_charizard_mewtwo_silver.png</t>
   </si>
   <si>
+    <t>pikachu charizard mewtwo silver</t>
+  </si>
+  <si>
     <t>coin_pikachu_gold.png</t>
   </si>
   <si>
+    <t>pikachu gold</t>
+  </si>
+  <si>
     <t>coin_pikachu_gold_1.png</t>
   </si>
   <si>
+    <t>pikachu gold 1</t>
+  </si>
+  <si>
     <t>coin_pikachu_gold_2.png</t>
   </si>
   <si>
+    <t>pikachu gold 2</t>
+  </si>
+  <si>
     <t>coin_pikachu_gold_3.png</t>
   </si>
   <si>
+    <t>pikachu gold 3</t>
+  </si>
+  <si>
+    <t>GAMBLER MICK</t>
+  </si>
+  <si>
     <t>coin_pikachu_red_1.png</t>
   </si>
   <si>
+    <t>pikachu red 1</t>
+  </si>
+  <si>
     <t>coin_pikachu_silver_1.png</t>
   </si>
   <si>
+    <t>pikachu silver 1</t>
+  </si>
+  <si>
+    <t>BEACH KID TIMOTHY</t>
+  </si>
+  <si>
     <t>coin_pikachu_silver_2.png</t>
   </si>
   <si>
+    <t>pikachu silver 2</t>
+  </si>
+  <si>
     <t>coin_piplup_blue.png</t>
   </si>
   <si>
+    <t>piplup blue</t>
+  </si>
+  <si>
     <t>coin_plasma_blue.png</t>
   </si>
   <si>
+    <t>plasma blue</t>
+  </si>
+  <si>
     <t>coin_plasma_silver.png</t>
   </si>
   <si>
+    <t>plasma silver</t>
+  </si>
+  <si>
     <t>coin_pokeball_red.png</t>
   </si>
   <si>
+    <t>pokeball red</t>
+  </si>
+  <si>
     <t>coin_popplio_blue.png</t>
   </si>
   <si>
+    <t>popplio blue</t>
+  </si>
+  <si>
     <t>coin_primal_groudon_red.png</t>
   </si>
   <si>
+    <t>primal groudon red</t>
+  </si>
+  <si>
     <t>coin_primal_kyogre_blue.png</t>
   </si>
   <si>
+    <t>primal kyogre blue</t>
+  </si>
+  <si>
     <t>coin_raichu_gold.png</t>
   </si>
   <si>
+    <t>raichu gold</t>
+  </si>
+  <si>
     <t>coin_raichu_gold_2.png</t>
   </si>
   <si>
+    <t>raichu gold 2</t>
+  </si>
+  <si>
     <t>coin_raikou_gold.png</t>
   </si>
   <si>
+    <t>raikou gold</t>
+  </si>
+  <si>
     <t>coin_rayquaza_gold.png</t>
   </si>
   <si>
+    <t>rayquaza gold</t>
+  </si>
+  <si>
     <t>coin_rayquaza_green.png</t>
   </si>
   <si>
+    <t>rayquaza green</t>
+  </si>
+  <si>
     <t>coin_rayquaza_silver.png</t>
   </si>
   <si>
+    <t>rayquaza silver</t>
+  </si>
+  <si>
+    <t>CARD ELDER HAMISH</t>
+  </si>
+  <si>
     <t>coin_reshiram_zekrom_silver.png</t>
   </si>
   <si>
+    <t>reshiram zekrom silver</t>
+  </si>
+  <si>
+    <t>BAD DUDE PAUL</t>
+  </si>
+  <si>
+    <t>coin_rocket_blue.png</t>
+  </si>
+  <si>
+    <t>rocket blue</t>
+  </si>
+  <si>
+    <t>ROCKET GRUNT DAMIEN</t>
+  </si>
+  <si>
+    <t>coin_rocket_red.png</t>
+  </si>
+  <si>
+    <t>rocket red</t>
+  </si>
+  <si>
+    <t>ROCKET GRUNT PENNY</t>
+  </si>
+  <si>
     <t>coin_rocket_silver.png</t>
   </si>
   <si>
+    <t>rocket silver</t>
+  </si>
+  <si>
     <t>coin_rowlett_green.png</t>
   </si>
   <si>
+    <t>rowlett green</t>
+  </si>
+  <si>
     <t>coin_salamance_gold.png</t>
   </si>
   <si>
+    <t>salamance gold</t>
+  </si>
+  <si>
     <t>coin_sceptile_green.png</t>
   </si>
   <si>
+    <t>sceptile green</t>
+  </si>
+  <si>
     <t>coin_scorbunny_red.png</t>
   </si>
   <si>
+    <t>scorbunny red</t>
+  </si>
+  <si>
+    <t>JOGGER DANIEL</t>
+  </si>
+  <si>
     <t>coin_sirfetchd_green.png</t>
   </si>
   <si>
+    <t>sirfetchd green</t>
+  </si>
+  <si>
     <t>coin_slowpoke_pink.png</t>
   </si>
   <si>
+    <t>slowpoke pink</t>
+  </si>
+  <si>
     <t>coin_snom_blue.png</t>
   </si>
   <si>
+    <t>snom blue</t>
+  </si>
+  <si>
     <t>coin_sobble_blue.png</t>
   </si>
   <si>
+    <t>sobble blue</t>
+  </si>
+  <si>
     <t>coin_solgaleo_gold.png</t>
   </si>
   <si>
+    <t>solgaleo gold</t>
+  </si>
+  <si>
+    <t>GUITARIST HOWARD</t>
+  </si>
+  <si>
     <t>coin_sprigatito_silver.png</t>
   </si>
   <si>
+    <t>sprigatito silver</t>
+  </si>
+  <si>
     <t>coin_steelix_silver.png</t>
   </si>
   <si>
+    <t>steelix silver</t>
+  </si>
+  <si>
     <t>coin_suicune_silver.png</t>
   </si>
   <si>
+    <t>suicune silver</t>
+  </si>
+  <si>
     <t>coin_swampert_blue.png</t>
   </si>
   <si>
+    <t>swampert blue</t>
+  </si>
+  <si>
     <t>coin_sylveon_pink.png</t>
   </si>
   <si>
+    <t>sylveon pink</t>
+  </si>
+  <si>
     <t>coin_terapagos_blue.png</t>
   </si>
   <si>
+    <t>terapagos blue</t>
+  </si>
+  <si>
     <t>coin_togepi_cleffa_igglybuff_pink.png</t>
   </si>
   <si>
+    <t>togepi cleffa igglybuff pink</t>
+  </si>
+  <si>
     <t>coin_totodile_blue.png</t>
   </si>
   <si>
+    <t>totodile blue</t>
+  </si>
+  <si>
     <t>coin_treeko_torchic_mudkip_silver.png</t>
   </si>
   <si>
+    <t>treeko torchic mudkip silver</t>
+  </si>
+  <si>
     <t>coin_turtwig_green.png</t>
   </si>
   <si>
+    <t>turtwig green</t>
+  </si>
+  <si>
     <t>coin_tyranitar_blue.png</t>
   </si>
   <si>
+    <t>tyranitar blue</t>
+  </si>
+  <si>
+    <t>coin_tyranitar_gold.png</t>
+  </si>
+  <si>
+    <t>tyranitar gold</t>
+  </si>
+  <si>
+    <t>HIKER BEN</t>
+  </si>
+  <si>
     <t>coin_tyranitar_silver.png</t>
   </si>
   <si>
+    <t>tyranitar silver</t>
+  </si>
+  <si>
     <t>coin_umbreon_black.png</t>
   </si>
   <si>
+    <t>umbreon black</t>
+  </si>
+  <si>
     <t>coin_umbreon_pink.png</t>
   </si>
   <si>
+    <t>umbreon pink</t>
+  </si>
+  <si>
     <t>coin_urshifu_blue.png</t>
   </si>
   <si>
+    <t>urshifu blue</t>
+  </si>
+  <si>
     <t>coin_urshifu_red.png</t>
   </si>
   <si>
+    <t>urshifu red</t>
+  </si>
+  <si>
     <t>coin_vaporeon_silver.png</t>
   </si>
   <si>
+    <t>vaporeon silver</t>
+  </si>
+  <si>
     <t>coin_venusaur_green.png</t>
   </si>
   <si>
+    <t>venusaur green</t>
+  </si>
+  <si>
+    <t>GARDEN MANAGER LOUIS</t>
+  </si>
+  <si>
     <t>coin_volcanion_red.png</t>
   </si>
   <si>
+    <t>volcanion red</t>
+  </si>
+  <si>
     <t>coin_wooloo_silver.png</t>
   </si>
   <si>
+    <t>wooloo silver</t>
+  </si>
+  <si>
     <t>coin_xerneas_blue.png</t>
   </si>
   <si>
+    <t>xerneas blue</t>
+  </si>
+  <si>
     <t>coin_xerneas_silver.png</t>
   </si>
   <si>
+    <t>xerneas silver</t>
+  </si>
+  <si>
     <t>coin_yampa_gold.png</t>
   </si>
   <si>
+    <t>yampa gold</t>
+  </si>
+  <si>
+    <t>SUNBATHING COIN GIVER</t>
+  </si>
+  <si>
     <t>coin_yveltal_red.png</t>
   </si>
   <si>
+    <t>yveltal red</t>
+  </si>
+  <si>
     <t>coin_yveltal_silver.png</t>
   </si>
   <si>
+    <t>yveltal silver</t>
+  </si>
+  <si>
     <t>coin_zapdos_gold.png</t>
   </si>
   <si>
+    <t>zapdos gold</t>
+  </si>
+  <si>
+    <t>GUITARIST JONESY</t>
+  </si>
+  <si>
     <t>coin_zoroark_silver.png</t>
   </si>
   <si>
-    <t>Coin</t>
-  </si>
-  <si>
-    <t>granted by name</t>
-  </si>
-  <si>
-    <t>granted day</t>
-  </si>
-  <si>
-    <t>Day 2</t>
-  </si>
-  <si>
-    <t>Firebreather Kenneth</t>
-  </si>
-  <si>
-    <t>Gardener Callum</t>
-  </si>
-  <si>
-    <t>Evening 1</t>
-  </si>
-  <si>
-    <t>Schoolboy_Adam</t>
-  </si>
-  <si>
-    <t>Day 1</t>
-  </si>
-  <si>
-    <t>Painter Jericho</t>
-  </si>
-  <si>
-    <t>Youngster Joey</t>
-  </si>
-  <si>
-    <t>Engineer Allan</t>
-  </si>
-  <si>
-    <t>Fisherman Dave</t>
-  </si>
-  <si>
-    <t>Fisherman John</t>
-  </si>
-  <si>
-    <t>Gambler Mick</t>
-  </si>
-  <si>
-    <t>Swimmer Jordan</t>
-  </si>
-  <si>
-    <t>Swimmer Todd</t>
-  </si>
-  <si>
-    <t>Battlegirl Sofia</t>
-  </si>
-  <si>
-    <t>Sailor Bob</t>
-  </si>
-  <si>
-    <t>Bug Catcher Johnny</t>
-  </si>
-  <si>
-    <t>Bug Catcher Alex</t>
-  </si>
-  <si>
-    <t>Psychic Brienne</t>
-  </si>
-  <si>
-    <t>FireBreather Darryl</t>
-  </si>
-  <si>
-    <t>Beach Kid Evie</t>
-  </si>
-  <si>
-    <t>Beach Kid Timothy</t>
-  </si>
-  <si>
-    <t>Sunbathing coin giver</t>
-  </si>
-  <si>
-    <t>Jogger Daniel</t>
-  </si>
-  <si>
-    <t>Evening 2</t>
-  </si>
-  <si>
-    <t>Bad Dude Paul</t>
-  </si>
-  <si>
-    <t>Coin Shop</t>
-  </si>
-  <si>
-    <t>Day 3+</t>
-  </si>
-  <si>
-    <t>Juice Bar</t>
-  </si>
-  <si>
-    <t>Day 2+</t>
-  </si>
-  <si>
-    <t>Day 3</t>
-  </si>
-  <si>
-    <t>Birdspotter Gregg</t>
-  </si>
-  <si>
-    <t>Swimmer Melissa</t>
-  </si>
-  <si>
-    <t>Bug Catcher Frankie</t>
-  </si>
-  <si>
-    <t>coin_gyarados_gold.png</t>
-  </si>
-  <si>
-    <t>Fisherman Gary</t>
-  </si>
-  <si>
-    <t>SS Anne Tourist Edmund</t>
-  </si>
-  <si>
-    <t>SS Anne Tourist Alissa</t>
-  </si>
-  <si>
-    <t>Guitarist Jonesy</t>
-  </si>
-  <si>
-    <t>Birdspotter Tamsin</t>
-  </si>
-  <si>
-    <t>Guitarist Howard</t>
-  </si>
-  <si>
-    <t>Young Twin Nella</t>
-  </si>
-  <si>
-    <t>Young Twin Anna</t>
-  </si>
-  <si>
-    <t>Garden Manager Louis</t>
-  </si>
-  <si>
-    <t>Card Elder Rayne</t>
-  </si>
-  <si>
-    <t>Day 3-4</t>
-  </si>
-  <si>
-    <t>Card Elder Waverly</t>
-  </si>
-  <si>
-    <t>Card Elder Hamish</t>
-  </si>
-  <si>
-    <t>coin_tyranitar_gold.png</t>
-  </si>
-  <si>
-    <t>Coin Name</t>
-  </si>
-  <si>
-    <t>alakazam purple</t>
-  </si>
-  <si>
-    <t>arcanine red</t>
-  </si>
-  <si>
-    <t>arceus silver</t>
-  </si>
-  <si>
-    <t>back basic</t>
-  </si>
-  <si>
-    <t>blastoise blue</t>
-  </si>
-  <si>
-    <t>blastoise blue 2</t>
-  </si>
-  <si>
-    <t>blastoise silver</t>
-  </si>
-  <si>
-    <t>bulbasaur green</t>
-  </si>
-  <si>
-    <t>celebi green</t>
-  </si>
-  <si>
-    <t>chansey green</t>
-  </si>
-  <si>
-    <t>chansey pink</t>
-  </si>
-  <si>
-    <t>chansey silver</t>
-  </si>
-  <si>
-    <t>charizard blue</t>
-  </si>
-  <si>
-    <t>charizard gold</t>
-  </si>
-  <si>
-    <t>charizard red</t>
-  </si>
-  <si>
-    <t>charizard silver</t>
-  </si>
-  <si>
-    <t>chespin silver</t>
-  </si>
-  <si>
-    <t>chikorita green</t>
-  </si>
-  <si>
-    <t>chimchar red</t>
-  </si>
-  <si>
-    <t>corviknight silver</t>
-  </si>
-  <si>
-    <t>crobat pink</t>
-  </si>
-  <si>
-    <t>cyndaquil red</t>
-  </si>
-  <si>
-    <t>darkrai gold</t>
-  </si>
-  <si>
-    <t>darkrai silver</t>
-  </si>
-  <si>
-    <t>darkrai umbreon silver</t>
-  </si>
-  <si>
-    <t>darmanitan blue</t>
-  </si>
-  <si>
-    <t>deoxys espeon silver</t>
-  </si>
-  <si>
-    <t>deoxys red</t>
-  </si>
-  <si>
-    <t>deoxys red 2</t>
-  </si>
-  <si>
-    <t>deoxys silver</t>
-  </si>
-  <si>
-    <t>dialga blue</t>
-  </si>
-  <si>
-    <t>dialga blue 2</t>
-  </si>
-  <si>
-    <t>dialga blue 3</t>
-  </si>
-  <si>
-    <t>dialga silver</t>
-  </si>
-  <si>
-    <t>dragonite gold</t>
-  </si>
-  <si>
-    <t>dragonite gold 2</t>
-  </si>
-  <si>
-    <t>eevee blue</t>
-  </si>
-  <si>
-    <t>eevee blue 2</t>
-  </si>
-  <si>
-    <t>eevee gold</t>
-  </si>
-  <si>
-    <t>eevee gold 2</t>
-  </si>
-  <si>
-    <t>eevee pink</t>
-  </si>
-  <si>
-    <t>eevee red</t>
-  </si>
-  <si>
-    <t>eevee silver</t>
-  </si>
-  <si>
-    <t>empoleon blue</t>
-  </si>
-  <si>
-    <t>energy black</t>
-  </si>
-  <si>
-    <t>energy black 2</t>
-  </si>
-  <si>
-    <t>energy blue</t>
-  </si>
-  <si>
-    <t>energy blue 2</t>
-  </si>
-  <si>
-    <t>energy brown</t>
-  </si>
-  <si>
-    <t>energy brown 2</t>
-  </si>
-  <si>
-    <t>energy gold</t>
-  </si>
-  <si>
-    <t>energy gold 2</t>
-  </si>
-  <si>
-    <t>energy gold 3</t>
-  </si>
-  <si>
-    <t>energy green</t>
-  </si>
-  <si>
-    <t>energy green 2</t>
-  </si>
-  <si>
-    <t>energy pink</t>
-  </si>
-  <si>
-    <t>energy purple</t>
-  </si>
-  <si>
-    <t>energy purple 2</t>
-  </si>
-  <si>
-    <t>energy red</t>
-  </si>
-  <si>
-    <t>energy red2</t>
-  </si>
-  <si>
-    <t>energy silver</t>
-  </si>
-  <si>
-    <t>energy silver 2</t>
-  </si>
-  <si>
-    <t>entei red</t>
-  </si>
-  <si>
-    <t>espeon pink</t>
-  </si>
-  <si>
-    <t>espeon purple</t>
-  </si>
-  <si>
-    <t>fennekin silver</t>
-  </si>
-  <si>
-    <t>flareon red</t>
-  </si>
-  <si>
-    <t>flygon green</t>
-  </si>
-  <si>
-    <t>froakie chespin fennekin silver</t>
-  </si>
-  <si>
-    <t>froakie silver</t>
-  </si>
-  <si>
-    <t>garchomp gold</t>
-  </si>
-  <si>
-    <t>gardevoir purple</t>
-  </si>
-  <si>
-    <t>gardevoir silver</t>
-  </si>
-  <si>
-    <t>gardevoir silver 2</t>
-  </si>
-  <si>
-    <t>genesect purple</t>
-  </si>
-  <si>
-    <t>genesect silver</t>
-  </si>
-  <si>
-    <t>glaceon blue</t>
-  </si>
-  <si>
-    <t>gloom green</t>
-  </si>
-  <si>
-    <t>grookey green</t>
-  </si>
-  <si>
-    <t>groudon red</t>
-  </si>
-  <si>
-    <t>gyarados blue</t>
-  </si>
-  <si>
-    <t>gyarados gold</t>
-  </si>
-  <si>
-    <t>gyarados red</t>
-  </si>
-  <si>
-    <t>hydreigon silver</t>
-  </si>
-  <si>
-    <t>infernape gallade gold</t>
-  </si>
-  <si>
-    <t>jigglypuff pink</t>
-  </si>
-  <si>
-    <t>jirachi gold</t>
-  </si>
-  <si>
-    <t>jolteon silver</t>
-  </si>
-  <si>
-    <t>koraidon red</t>
-  </si>
-  <si>
-    <t>kyogre blue</t>
-  </si>
-  <si>
-    <t>leafeon green</t>
-  </si>
-  <si>
-    <t>litten red</t>
-  </si>
-  <si>
-    <t>lucario gold</t>
-  </si>
-  <si>
-    <t>lucario red</t>
-  </si>
-  <si>
-    <t>lugia silver</t>
-  </si>
-  <si>
-    <t>lunala purple</t>
-  </si>
-  <si>
-    <t>magmortar electrivire gold</t>
-  </si>
-  <si>
-    <t>magmortar electrivire red</t>
-  </si>
-  <si>
-    <t>manaphy blue</t>
-  </si>
-  <si>
-    <t>melmetal silver</t>
-  </si>
-  <si>
-    <t>metagross silver</t>
-  </si>
-  <si>
-    <t>mewtwo purple</t>
-  </si>
-  <si>
-    <t>mewtwo purple 2</t>
-  </si>
-  <si>
-    <t>mew blue</t>
-  </si>
-  <si>
-    <t>mew pink</t>
-  </si>
-  <si>
-    <t>mew pink 2</t>
-  </si>
-  <si>
-    <t>mew silver</t>
-  </si>
-  <si>
-    <t>miraidon purple</t>
-  </si>
-  <si>
-    <t>munchlax gold</t>
-  </si>
-  <si>
-    <t>munchlax silver</t>
-  </si>
-  <si>
-    <t>ninetales red</t>
-  </si>
-  <si>
-    <t>ninetales silver</t>
-  </si>
-  <si>
-    <t>onix brown</t>
-  </si>
-  <si>
-    <t>palkia pink 1</t>
-  </si>
-  <si>
-    <t>palkia pink 2</t>
-  </si>
-  <si>
-    <t>palkia pink 3</t>
-  </si>
-  <si>
-    <t>palkia silver</t>
-  </si>
-  <si>
-    <t>pichu gold</t>
-  </si>
-  <si>
-    <t>pikachu charizard mewtwo silver</t>
-  </si>
-  <si>
-    <t>pikachu gold</t>
-  </si>
-  <si>
-    <t>pikachu gold 1</t>
-  </si>
-  <si>
-    <t>pikachu gold 2</t>
-  </si>
-  <si>
-    <t>pikachu gold 3</t>
-  </si>
-  <si>
-    <t>pikachu red 1</t>
-  </si>
-  <si>
-    <t>pikachu silver 1</t>
-  </si>
-  <si>
-    <t>pikachu silver 2</t>
-  </si>
-  <si>
-    <t>piplup blue</t>
-  </si>
-  <si>
-    <t>plasma blue</t>
-  </si>
-  <si>
-    <t>plasma silver</t>
-  </si>
-  <si>
-    <t>pokeball red</t>
-  </si>
-  <si>
-    <t>popplio blue</t>
-  </si>
-  <si>
-    <t>primal groudon red</t>
-  </si>
-  <si>
-    <t>primal kyogre blue</t>
-  </si>
-  <si>
-    <t>raichu gold</t>
-  </si>
-  <si>
-    <t>raichu gold 2</t>
-  </si>
-  <si>
-    <t>raikou gold</t>
-  </si>
-  <si>
-    <t>rayquaza gold</t>
-  </si>
-  <si>
-    <t>rayquaza green</t>
-  </si>
-  <si>
-    <t>rayquaza silver</t>
-  </si>
-  <si>
-    <t>reshiram zekrom silver</t>
-  </si>
-  <si>
-    <t>rocket silver</t>
-  </si>
-  <si>
-    <t>rowlett green</t>
-  </si>
-  <si>
-    <t>salamance gold</t>
-  </si>
-  <si>
-    <t>sceptile green</t>
-  </si>
-  <si>
-    <t>scorbunny red</t>
-  </si>
-  <si>
-    <t>sirfetchd green</t>
-  </si>
-  <si>
-    <t>slowpoke pink</t>
-  </si>
-  <si>
-    <t>snom blue</t>
-  </si>
-  <si>
-    <t>sobble blue</t>
-  </si>
-  <si>
-    <t>solgaleo gold</t>
-  </si>
-  <si>
-    <t>sprigatito silver</t>
-  </si>
-  <si>
-    <t>steelix silver</t>
-  </si>
-  <si>
-    <t>suicune silver</t>
-  </si>
-  <si>
-    <t>swampert blue</t>
-  </si>
-  <si>
-    <t>sylveon pink</t>
-  </si>
-  <si>
-    <t>terapagos blue</t>
-  </si>
-  <si>
-    <t>togepi cleffa igglybuff pink</t>
-  </si>
-  <si>
-    <t>totodile blue</t>
-  </si>
-  <si>
-    <t>treeko torchic mudkip silver</t>
-  </si>
-  <si>
-    <t>turtwig green</t>
-  </si>
-  <si>
-    <t>tyranitar blue</t>
-  </si>
-  <si>
-    <t>tyranitar gold</t>
-  </si>
-  <si>
-    <t>tyranitar silver</t>
-  </si>
-  <si>
-    <t>umbreon black</t>
-  </si>
-  <si>
-    <t>umbreon pink</t>
-  </si>
-  <si>
-    <t>urshifu blue</t>
-  </si>
-  <si>
-    <t>urshifu red</t>
-  </si>
-  <si>
-    <t>vaporeon silver</t>
-  </si>
-  <si>
-    <t>venusaur green</t>
-  </si>
-  <si>
-    <t>volcanion red</t>
-  </si>
-  <si>
-    <t>wooloo silver</t>
-  </si>
-  <si>
-    <t>xerneas blue</t>
-  </si>
-  <si>
-    <t>xerneas silver</t>
-  </si>
-  <si>
-    <t>yampa gold</t>
-  </si>
-  <si>
-    <t>yveltal red</t>
-  </si>
-  <si>
-    <t>yveltal silver</t>
-  </si>
-  <si>
-    <t>zapdos gold</t>
-  </si>
-  <si>
     <t>zoroark silver</t>
   </si>
   <si>
-    <t>Hiker Ben</t>
-  </si>
-  <si>
-    <t>Evening 3</t>
-  </si>
-  <si>
-    <t>Bad Dude Wayne</t>
-  </si>
-  <si>
-    <t>Night 3</t>
-  </si>
-  <si>
-    <t>rocket blue</t>
-  </si>
-  <si>
-    <t>rocket red</t>
-  </si>
-  <si>
-    <t>Rocket Grunt Damien</t>
-  </si>
-  <si>
-    <t>Rocket Grunt Penny</t>
+    <t>BAD DUDE WAYNE</t>
   </si>
 </sst>
 </file>
@@ -1335,13 +1334,11 @@
     <dxf>
       <font>
         <b/>
-        <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
@@ -1364,16 +1361,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CABA093D-E10D-4AFA-84B7-B1B7EB5F6B16}" name="Table1" displayName="Table1" ref="A1:D181" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:D181" xr:uid="{CABA093D-E10D-4AFA-84B7-B1B7EB5F6B16}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D181" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D181" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:D179">
     <sortCondition ref="C1:C181"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{B1B3F4BF-11CF-4DCD-BBFF-800CA95AB652}" name="Coin"/>
-    <tableColumn id="4" xr3:uid="{F48141CC-50B0-4B5B-B36E-7B26E2763CED}" name="Coin Name"/>
-    <tableColumn id="2" xr3:uid="{2B45EC9D-2894-4946-81C0-66214EF570D9}" name="granted by name"/>
-    <tableColumn id="3" xr3:uid="{7746DE0B-7B46-4C19-BAE4-2167203617DB}" name="granted day"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Coin"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Coin Name"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="granted by name"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="granted day"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1695,7 +1692,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E36B1B59-0D5E-4C8D-AEE2-CA809DBB4E7C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D181"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1707,1768 +1704,1807 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>176</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>228</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>177</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>178</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>229</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>230</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>180</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>231</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>232</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>233</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>234</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>235</v>
-      </c>
-      <c r="C8" t="s">
-        <v>223</v>
-      </c>
-      <c r="D8" t="s">
-        <v>224</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>236</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>181</v>
+        <v>26</v>
       </c>
       <c r="D9" t="s">
-        <v>182</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>237</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>238</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>221</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>209</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>239</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>220</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>209</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
-        <v>240</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>183</v>
+        <v>39</v>
       </c>
       <c r="D13" t="s">
-        <v>184</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B14" t="s">
-        <v>241</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B15" t="s">
-        <v>242</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>243</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s">
-        <v>244</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="B18" t="s">
-        <v>245</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>246</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="B20" t="s">
-        <v>247</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="B21" t="s">
-        <v>248</v>
+        <v>56</v>
       </c>
       <c r="C21" t="s">
-        <v>218</v>
+        <v>57</v>
       </c>
       <c r="D21" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="B22" t="s">
-        <v>249</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s">
-        <v>250</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>251</v>
+        <v>64</v>
+      </c>
+      <c r="C24" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="B25" t="s">
-        <v>252</v>
+        <v>66</v>
       </c>
       <c r="C25" t="s">
-        <v>409</v>
+        <v>419</v>
       </c>
       <c r="D25" t="s">
-        <v>410</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="B26" t="s">
-        <v>253</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="B27" t="s">
-        <v>254</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>255</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="B29" t="s">
-        <v>256</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="B30" t="s">
-        <v>257</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
       <c r="B31" t="s">
-        <v>258</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="B32" t="s">
-        <v>259</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="B33" t="s">
-        <v>260</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="B34" t="s">
-        <v>261</v>
+        <v>86</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>87</v>
       </c>
       <c r="B35" t="s">
-        <v>262</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="B36" t="s">
-        <v>263</v>
+        <v>90</v>
       </c>
       <c r="C36" t="s">
-        <v>215</v>
+        <v>91</v>
+      </c>
+      <c r="D36" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>92</v>
       </c>
       <c r="B37" t="s">
-        <v>264</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>94</v>
       </c>
       <c r="B38" t="s">
-        <v>265</v>
+        <v>95</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>96</v>
       </c>
       <c r="B39" t="s">
-        <v>266</v>
+        <v>97</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="B40" t="s">
-        <v>267</v>
+        <v>99</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="B41" t="s">
-        <v>268</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>102</v>
       </c>
       <c r="B42" t="s">
-        <v>269</v>
+        <v>103</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="B43" t="s">
-        <v>270</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="B44" t="s">
-        <v>271</v>
+        <v>107</v>
       </c>
       <c r="C44" t="s">
-        <v>185</v>
+        <v>108</v>
       </c>
       <c r="D44" t="s">
-        <v>182</v>
+        <v>27</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>43</v>
+        <v>109</v>
       </c>
       <c r="B45" t="s">
-        <v>272</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>111</v>
       </c>
       <c r="B46" t="s">
-        <v>273</v>
+        <v>112</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>113</v>
       </c>
       <c r="B47" t="s">
-        <v>274</v>
+        <v>114</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>46</v>
+        <v>115</v>
       </c>
       <c r="B48" t="s">
-        <v>275</v>
+        <v>116</v>
       </c>
       <c r="C48" t="s">
-        <v>191</v>
+        <v>117</v>
       </c>
       <c r="D48" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>47</v>
+        <v>118</v>
       </c>
       <c r="B49" t="s">
-        <v>276</v>
+        <v>119</v>
       </c>
       <c r="C49" t="s">
-        <v>192</v>
+        <v>120</v>
       </c>
       <c r="D49" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>48</v>
+        <v>121</v>
       </c>
       <c r="B50" t="s">
-        <v>277</v>
+        <v>122</v>
       </c>
       <c r="C50" t="s">
-        <v>193</v>
+        <v>123</v>
       </c>
       <c r="D50" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>49</v>
+        <v>124</v>
       </c>
       <c r="B51" t="s">
-        <v>278</v>
+        <v>125</v>
       </c>
       <c r="C51" t="s">
-        <v>194</v>
+        <v>126</v>
       </c>
       <c r="D51" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>50</v>
+        <v>127</v>
       </c>
       <c r="B52" t="s">
-        <v>279</v>
+        <v>128</v>
       </c>
       <c r="C52" t="s">
-        <v>187</v>
+        <v>129</v>
       </c>
       <c r="D52" t="s">
-        <v>182</v>
+        <v>27</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>51</v>
+        <v>130</v>
       </c>
       <c r="B53" t="s">
-        <v>280</v>
+        <v>131</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>52</v>
+        <v>132</v>
       </c>
       <c r="B54" t="s">
-        <v>281</v>
+        <v>133</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>53</v>
+        <v>134</v>
       </c>
       <c r="B55" t="s">
-        <v>282</v>
+        <v>135</v>
       </c>
       <c r="C55" t="s">
-        <v>196</v>
+        <v>136</v>
       </c>
       <c r="D55" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>54</v>
+        <v>137</v>
       </c>
       <c r="B56" t="s">
-        <v>283</v>
+        <v>138</v>
+      </c>
+      <c r="C56" t="s">
+        <v>139</v>
+      </c>
+      <c r="D56" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>55</v>
+        <v>140</v>
       </c>
       <c r="B57" t="s">
-        <v>284</v>
+        <v>141</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>56</v>
+        <v>142</v>
       </c>
       <c r="B58" t="s">
-        <v>285</v>
+        <v>143</v>
       </c>
       <c r="C58" t="s">
-        <v>197</v>
+        <v>144</v>
       </c>
       <c r="D58" t="s">
-        <v>179</v>
+        <v>68</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>57</v>
+        <v>145</v>
       </c>
       <c r="B59" t="s">
-        <v>286</v>
+        <v>146</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>58</v>
+        <v>147</v>
       </c>
       <c r="B60" t="s">
-        <v>287</v>
+        <v>148</v>
       </c>
       <c r="C60" t="s">
-        <v>198</v>
+        <v>149</v>
       </c>
       <c r="D60" t="s">
-        <v>179</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>59</v>
+        <v>150</v>
       </c>
       <c r="B61" t="s">
-        <v>288</v>
+        <v>151</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>60</v>
+        <v>152</v>
       </c>
       <c r="B62" t="s">
-        <v>289</v>
+        <v>153</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>61</v>
+        <v>154</v>
       </c>
       <c r="B63" t="s">
-        <v>290</v>
+        <v>155</v>
       </c>
       <c r="C63" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="D63" t="s">
-        <v>184</v>
+        <v>40</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>62</v>
+        <v>157</v>
       </c>
       <c r="B64" t="s">
-        <v>291</v>
+        <v>158</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>63</v>
+        <v>159</v>
       </c>
       <c r="B65" t="s">
-        <v>292</v>
+        <v>160</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>64</v>
+        <v>161</v>
       </c>
       <c r="B66" t="s">
-        <v>293</v>
+        <v>162</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="B67" t="s">
-        <v>294</v>
+        <v>164</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>66</v>
+        <v>165</v>
       </c>
       <c r="B68" t="s">
-        <v>295</v>
+        <v>166</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>67</v>
+        <v>167</v>
       </c>
       <c r="B69" t="s">
-        <v>296</v>
+        <v>168</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>68</v>
+        <v>169</v>
       </c>
       <c r="B70" t="s">
-        <v>297</v>
+        <v>170</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>69</v>
+        <v>171</v>
       </c>
       <c r="B71" t="s">
-        <v>298</v>
+        <v>172</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>70</v>
+        <v>173</v>
       </c>
       <c r="B72" t="s">
-        <v>299</v>
+        <v>174</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>71</v>
+        <v>175</v>
       </c>
       <c r="B73" t="s">
-        <v>300</v>
+        <v>176</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>72</v>
+        <v>177</v>
       </c>
       <c r="B74" t="s">
-        <v>301</v>
+        <v>178</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>73</v>
+        <v>179</v>
       </c>
       <c r="B75" t="s">
-        <v>302</v>
+        <v>180</v>
       </c>
       <c r="C75" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D75" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>74</v>
+        <v>181</v>
       </c>
       <c r="B76" t="s">
-        <v>303</v>
+        <v>182</v>
       </c>
       <c r="C76" t="s">
-        <v>212</v>
+        <v>183</v>
       </c>
       <c r="D76" t="s">
-        <v>209</v>
+        <v>33</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>75</v>
+        <v>184</v>
       </c>
       <c r="B77" t="s">
-        <v>304</v>
-      </c>
-      <c r="C77" t="s">
-        <v>225</v>
-      </c>
-      <c r="D77" t="s">
-        <v>224</v>
+        <v>185</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>76</v>
+        <v>187</v>
       </c>
       <c r="B78" t="s">
-        <v>305</v>
+        <v>188</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>77</v>
+        <v>189</v>
       </c>
       <c r="B79" t="s">
-        <v>306</v>
+        <v>190</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>78</v>
+        <v>191</v>
       </c>
       <c r="B80" t="s">
-        <v>307</v>
+        <v>192</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>79</v>
+        <v>193</v>
       </c>
       <c r="B81" t="s">
-        <v>308</v>
+        <v>194</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>80</v>
+        <v>195</v>
       </c>
       <c r="B82" t="s">
-        <v>309</v>
+        <v>196</v>
       </c>
       <c r="C82" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="D82" t="s">
-        <v>184</v>
+        <v>40</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="B83" t="s">
-        <v>310</v>
+        <v>199</v>
       </c>
       <c r="C83" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
       <c r="D83" t="s">
-        <v>209</v>
+        <v>33</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>81</v>
+        <v>201</v>
       </c>
       <c r="B84" t="s">
-        <v>311</v>
+        <v>202</v>
       </c>
       <c r="C84" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D84" t="s">
-        <v>184</v>
+        <v>27</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>82</v>
+        <v>204</v>
       </c>
       <c r="B85" t="s">
-        <v>312</v>
+        <v>205</v>
       </c>
       <c r="C85" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D85" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>83</v>
+        <v>206</v>
       </c>
       <c r="B86" t="s">
-        <v>313</v>
+        <v>207</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>84</v>
+        <v>208</v>
       </c>
       <c r="B87" t="s">
-        <v>314</v>
+        <v>209</v>
       </c>
       <c r="C87" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="D87" t="s">
-        <v>209</v>
+        <v>33</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>85</v>
+        <v>211</v>
       </c>
       <c r="B88" t="s">
-        <v>315</v>
+        <v>212</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>86</v>
+        <v>213</v>
       </c>
       <c r="B89" t="s">
-        <v>316</v>
+        <v>214</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>87</v>
+        <v>215</v>
       </c>
       <c r="B90" t="s">
-        <v>317</v>
+        <v>216</v>
+      </c>
+      <c r="C90" t="s">
+        <v>217</v>
+      </c>
+      <c r="D90" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>88</v>
+        <v>219</v>
       </c>
       <c r="B91" t="s">
-        <v>318</v>
+        <v>220</v>
       </c>
       <c r="C91" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="D91" t="s">
-        <v>209</v>
+        <v>33</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>89</v>
+        <v>222</v>
       </c>
       <c r="B92" t="s">
-        <v>319</v>
+        <v>223</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>90</v>
+        <v>224</v>
       </c>
       <c r="B93" t="s">
-        <v>320</v>
+        <v>225</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>91</v>
+        <v>226</v>
       </c>
       <c r="B94" t="s">
-        <v>321</v>
+        <v>227</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>92</v>
+        <v>228</v>
       </c>
       <c r="B95" t="s">
-        <v>322</v>
+        <v>229</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>93</v>
+        <v>230</v>
       </c>
       <c r="B96" t="s">
-        <v>323</v>
+        <v>231</v>
       </c>
       <c r="C96" t="s">
-        <v>210</v>
+        <v>232</v>
       </c>
       <c r="D96" t="s">
-        <v>209</v>
+        <v>33</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>94</v>
+        <v>233</v>
       </c>
       <c r="B97" t="s">
-        <v>324</v>
+        <v>234</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>95</v>
+        <v>235</v>
       </c>
       <c r="B98" t="s">
-        <v>325</v>
+        <v>236</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>96</v>
+        <v>237</v>
       </c>
       <c r="B99" t="s">
-        <v>326</v>
+        <v>238</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>97</v>
+        <v>239</v>
       </c>
       <c r="B100" t="s">
-        <v>327</v>
+        <v>240</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>98</v>
+        <v>241</v>
       </c>
       <c r="B101" t="s">
-        <v>328</v>
+        <v>242</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>99</v>
+        <v>243</v>
       </c>
       <c r="B102" t="s">
-        <v>329</v>
+        <v>244</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>100</v>
+        <v>245</v>
       </c>
       <c r="B103" t="s">
-        <v>330</v>
+        <v>246</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>101</v>
+        <v>247</v>
       </c>
       <c r="B104" t="s">
-        <v>331</v>
+        <v>248</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>102</v>
+        <v>249</v>
       </c>
       <c r="B105" t="s">
-        <v>332</v>
+        <v>250</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>103</v>
+        <v>251</v>
       </c>
       <c r="B106" t="s">
-        <v>333</v>
+        <v>252</v>
       </c>
       <c r="C106" t="s">
-        <v>199</v>
+        <v>253</v>
       </c>
       <c r="D106" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>104</v>
+        <v>254</v>
       </c>
       <c r="B107" t="s">
-        <v>334</v>
+        <v>255</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>105</v>
+        <v>256</v>
       </c>
       <c r="B108" t="s">
-        <v>335</v>
+        <v>257</v>
       </c>
       <c r="D108" t="s">
-        <v>209</v>
+        <v>33</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>106</v>
+        <v>258</v>
       </c>
       <c r="B109" t="s">
-        <v>336</v>
+        <v>259</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>107</v>
+        <v>260</v>
       </c>
       <c r="B110" t="s">
-        <v>337</v>
+        <v>261</v>
       </c>
       <c r="C110" t="s">
-        <v>207</v>
+        <v>262</v>
       </c>
       <c r="D110" t="s">
-        <v>208</v>
+        <v>263</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>108</v>
+        <v>264</v>
       </c>
       <c r="B111" t="s">
-        <v>338</v>
+        <v>265</v>
       </c>
       <c r="C111" t="s">
-        <v>207</v>
+        <v>262</v>
       </c>
       <c r="D111" t="s">
-        <v>208</v>
+        <v>263</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>109</v>
+        <v>266</v>
       </c>
       <c r="B112" t="s">
-        <v>339</v>
+        <v>267</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>110</v>
+        <v>268</v>
       </c>
       <c r="B113" t="s">
-        <v>340</v>
+        <v>269</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>111</v>
+        <v>270</v>
       </c>
       <c r="B114" t="s">
-        <v>341</v>
+        <v>271</v>
+      </c>
+      <c r="C114" t="s">
+        <v>272</v>
+      </c>
+      <c r="D114" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>112</v>
+        <v>273</v>
       </c>
       <c r="B115" t="s">
-        <v>342</v>
+        <v>274</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>113</v>
+        <v>275</v>
       </c>
       <c r="B116" t="s">
-        <v>343</v>
+        <v>276</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>114</v>
+        <v>277</v>
       </c>
       <c r="B117" t="s">
-        <v>344</v>
+        <v>278</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>115</v>
+        <v>279</v>
       </c>
       <c r="B118" t="s">
-        <v>345</v>
+        <v>280</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>116</v>
+        <v>281</v>
       </c>
       <c r="B119" t="s">
-        <v>346</v>
+        <v>282</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>117</v>
+        <v>283</v>
       </c>
       <c r="B120" t="s">
-        <v>347</v>
+        <v>284</v>
       </c>
       <c r="C120" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D120" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>118</v>
+        <v>285</v>
       </c>
       <c r="B121" t="s">
-        <v>348</v>
+        <v>286</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>119</v>
+        <v>287</v>
       </c>
       <c r="B122" t="s">
-        <v>349</v>
+        <v>288</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>120</v>
+        <v>289</v>
       </c>
       <c r="B123" t="s">
-        <v>350</v>
+        <v>290</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>121</v>
+        <v>291</v>
       </c>
       <c r="B124" t="s">
-        <v>351</v>
+        <v>292</v>
       </c>
       <c r="C124" t="s">
-        <v>190</v>
+        <v>293</v>
       </c>
       <c r="D124" t="s">
-        <v>184</v>
+        <v>40</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>122</v>
+        <v>294</v>
       </c>
       <c r="B125" t="s">
-        <v>352</v>
+        <v>295</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>123</v>
+        <v>296</v>
       </c>
       <c r="B126" t="s">
-        <v>353</v>
+        <v>297</v>
       </c>
       <c r="C126" t="s">
-        <v>200</v>
+        <v>298</v>
       </c>
       <c r="D126" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>124</v>
+        <v>299</v>
       </c>
       <c r="B127" t="s">
-        <v>354</v>
+        <v>300</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>125</v>
+        <v>301</v>
       </c>
       <c r="B128" t="s">
-        <v>355</v>
+        <v>302</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>126</v>
+        <v>303</v>
       </c>
       <c r="B129" t="s">
-        <v>356</v>
+        <v>304</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>127</v>
+        <v>305</v>
       </c>
       <c r="B130" t="s">
-        <v>357</v>
+        <v>306</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>128</v>
+        <v>307</v>
       </c>
       <c r="B131" t="s">
-        <v>358</v>
+        <v>308</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>129</v>
+        <v>309</v>
       </c>
       <c r="B132" t="s">
-        <v>359</v>
+        <v>310</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>130</v>
+        <v>311</v>
       </c>
       <c r="B133" t="s">
-        <v>360</v>
+        <v>312</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>131</v>
+        <v>313</v>
       </c>
       <c r="B134" t="s">
-        <v>361</v>
+        <v>314</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>132</v>
+        <v>315</v>
       </c>
       <c r="B135" t="s">
-        <v>362</v>
+        <v>316</v>
+      </c>
+      <c r="C135" t="s">
+        <v>217</v>
+      </c>
+      <c r="D135" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>133</v>
+        <v>317</v>
       </c>
       <c r="B136" t="s">
-        <v>363</v>
+        <v>318</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>134</v>
+        <v>319</v>
       </c>
       <c r="B137" t="s">
-        <v>364</v>
+        <v>320</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>135</v>
+        <v>321</v>
       </c>
       <c r="B138" t="s">
-        <v>365</v>
+        <v>322</v>
+      </c>
+      <c r="C138" t="s">
+        <v>186</v>
+      </c>
+      <c r="D138" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>136</v>
+        <v>323</v>
       </c>
       <c r="B139" t="s">
-        <v>366</v>
+        <v>324</v>
+      </c>
+      <c r="C139" t="s">
+        <v>327</v>
+      </c>
+      <c r="D139" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>137</v>
+        <v>325</v>
       </c>
       <c r="B140" t="s">
-        <v>367</v>
+        <v>326</v>
       </c>
       <c r="C140" t="s">
-        <v>226</v>
+        <v>22</v>
       </c>
       <c r="D140" t="s">
-        <v>224</v>
+        <v>23</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>138</v>
+        <v>328</v>
       </c>
       <c r="B141" t="s">
-        <v>368</v>
+        <v>329</v>
       </c>
       <c r="C141" t="s">
-        <v>204</v>
+        <v>330</v>
       </c>
       <c r="D141" t="s">
-        <v>203</v>
+        <v>68</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>331</v>
+      </c>
       <c r="B142" t="s">
-        <v>411</v>
+        <v>332</v>
       </c>
       <c r="C142" t="s">
-        <v>413</v>
+        <v>333</v>
       </c>
       <c r="D142" t="s">
-        <v>410</v>
+        <v>218</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>334</v>
+      </c>
       <c r="B143" t="s">
-        <v>412</v>
+        <v>335</v>
       </c>
       <c r="C143" t="s">
-        <v>414</v>
+        <v>336</v>
       </c>
       <c r="D143" t="s">
-        <v>410</v>
+        <v>218</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>139</v>
+        <v>337</v>
       </c>
       <c r="B144" t="s">
-        <v>369</v>
+        <v>338</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>140</v>
+        <v>339</v>
       </c>
       <c r="B145" t="s">
-        <v>370</v>
+        <v>340</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>141</v>
+        <v>341</v>
       </c>
       <c r="B146" t="s">
-        <v>371</v>
+        <v>342</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>142</v>
+        <v>343</v>
       </c>
       <c r="B147" t="s">
-        <v>372</v>
+        <v>344</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>143</v>
+        <v>345</v>
       </c>
       <c r="B148" t="s">
-        <v>373</v>
+        <v>346</v>
       </c>
       <c r="C148" t="s">
-        <v>202</v>
+        <v>347</v>
       </c>
       <c r="D148" t="s">
-        <v>203</v>
+        <v>9</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>144</v>
+        <v>348</v>
       </c>
       <c r="B149" t="s">
-        <v>374</v>
+        <v>349</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>145</v>
+        <v>350</v>
       </c>
       <c r="B150" t="s">
-        <v>375</v>
+        <v>351</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>146</v>
+        <v>352</v>
       </c>
       <c r="B151" t="s">
-        <v>376</v>
+        <v>353</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>147</v>
+        <v>354</v>
       </c>
       <c r="B152" t="s">
-        <v>377</v>
+        <v>355</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>148</v>
+        <v>356</v>
       </c>
       <c r="B153" t="s">
-        <v>378</v>
+        <v>357</v>
       </c>
       <c r="C153" t="s">
-        <v>219</v>
+        <v>358</v>
       </c>
       <c r="D153" t="s">
-        <v>209</v>
+        <v>23</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>149</v>
+        <v>359</v>
       </c>
       <c r="B154" t="s">
-        <v>379</v>
+        <v>360</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>150</v>
+        <v>361</v>
       </c>
       <c r="B155" t="s">
-        <v>380</v>
+        <v>362</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>151</v>
+        <v>363</v>
       </c>
       <c r="B156" t="s">
-        <v>381</v>
+        <v>364</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>152</v>
+        <v>365</v>
       </c>
       <c r="B157" t="s">
-        <v>382</v>
+        <v>366</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>153</v>
+        <v>367</v>
       </c>
       <c r="B158" t="s">
-        <v>383</v>
+        <v>368</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>154</v>
+        <v>369</v>
       </c>
       <c r="B159" t="s">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="C159" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D159" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>155</v>
+        <v>371</v>
       </c>
       <c r="B160" t="s">
-        <v>385</v>
+        <v>372</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>156</v>
+        <v>373</v>
       </c>
       <c r="B161" t="s">
-        <v>386</v>
+        <v>374</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>157</v>
+        <v>375</v>
       </c>
       <c r="B162" t="s">
-        <v>387</v>
+        <v>376</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>158</v>
+        <v>377</v>
       </c>
       <c r="B163" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="C163" t="s">
-        <v>195</v>
+        <v>139</v>
       </c>
       <c r="D163" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>159</v>
+        <v>379</v>
       </c>
       <c r="B164" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>227</v>
+        <v>381</v>
       </c>
       <c r="B165" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="C165" t="s">
-        <v>407</v>
+        <v>383</v>
       </c>
       <c r="D165" t="s">
-        <v>408</v>
+        <v>23</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>160</v>
+        <v>384</v>
       </c>
       <c r="B166" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>161</v>
+        <v>386</v>
       </c>
       <c r="B167" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>162</v>
+        <v>388</v>
       </c>
       <c r="B168" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>163</v>
+        <v>390</v>
       </c>
       <c r="B169" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="C169" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D169" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>164</v>
+        <v>392</v>
       </c>
       <c r="B170" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C170" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D170" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>165</v>
+        <v>394</v>
       </c>
       <c r="B171" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>166</v>
+        <v>396</v>
       </c>
       <c r="B172" t="s">
         <v>397</v>
       </c>
       <c r="C172" t="s">
-        <v>222</v>
+        <v>398</v>
       </c>
       <c r="D172" t="s">
-        <v>209</v>
+        <v>23</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>167</v>
+        <v>399</v>
       </c>
       <c r="B173" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>168</v>
+        <v>401</v>
       </c>
       <c r="B174" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="C174" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D174" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>169</v>
+        <v>403</v>
       </c>
       <c r="B175" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>170</v>
+        <v>405</v>
       </c>
       <c r="B176" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="C176" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D176" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>171</v>
+        <v>407</v>
       </c>
       <c r="B177" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="C177" t="s">
-        <v>201</v>
+        <v>409</v>
       </c>
       <c r="D177" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>172</v>
+        <v>410</v>
       </c>
       <c r="B178" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>173</v>
+        <v>412</v>
       </c>
       <c r="B179" t="s">
-        <v>404</v>
+        <v>413</v>
       </c>
       <c r="C179" t="s">
-        <v>205</v>
+        <v>12</v>
       </c>
       <c r="D179" t="s">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>174</v>
+        <v>414</v>
       </c>
       <c r="B180" t="s">
-        <v>405</v>
+        <v>415</v>
       </c>
       <c r="C180" t="s">
-        <v>217</v>
+        <v>416</v>
       </c>
       <c r="D180" t="s">
-        <v>209</v>
+        <v>23</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>175</v>
+        <v>417</v>
       </c>
       <c r="B181" t="s">
-        <v>406</v>
+        <v>418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Created Verdant Harbour NPC file with Pikachu Kids
</commit_message>
<xml_diff>
--- a/Coin_tracker.xlsx
+++ b/Coin_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34EF1D5-10FB-4372-A8A7-65986C101030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C7951E-B1C6-47D3-A167-7DE97DA28B99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="23385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="430">
   <si>
     <t>Coin</t>
   </si>
@@ -907,9 +907,6 @@
     <t>coin_pikachu_red_1.png</t>
   </si>
   <si>
-    <t>pikachu red 1</t>
-  </si>
-  <si>
     <t>coin_pikachu_silver_1.png</t>
   </si>
   <si>
@@ -1280,6 +1277,39 @@
   </si>
   <si>
     <t>BAD DUDE WAYNE</t>
+  </si>
+  <si>
+    <t>pikachu red</t>
+  </si>
+  <si>
+    <t>pikachu blue</t>
+  </si>
+  <si>
+    <t>pikachu gold 4</t>
+  </si>
+  <si>
+    <t>Pikachu Fan Marina</t>
+  </si>
+  <si>
+    <t>Pikachu Fan Cami</t>
+  </si>
+  <si>
+    <t>Pikachu Fan Skye</t>
+  </si>
+  <si>
+    <t>Pikachu Fan Juniper</t>
+  </si>
+  <si>
+    <t>Pikachy Fan Leaf</t>
+  </si>
+  <si>
+    <t>Day 4</t>
+  </si>
+  <si>
+    <t>Pikachu Fan Raye</t>
+  </si>
+  <si>
+    <t>Pikachu Mum</t>
   </si>
 </sst>
 </file>
@@ -1361,10 +1391,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D181" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:D181" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:D179">
-    <sortCondition ref="C1:C181"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D183" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D183" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:D181">
+    <sortCondition ref="C1:C183"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Coin"/>
@@ -1693,7 +1723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D181"/>
+  <dimension ref="A1:D183"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" hidden="1" customWidth="1"/>
@@ -1956,7 +1986,7 @@
         <v>66</v>
       </c>
       <c r="C25" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D25" t="s">
         <v>218</v>
@@ -2888,196 +2918,217 @@
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>285</v>
-      </c>
       <c r="B121" t="s">
-        <v>286</v>
+        <v>420</v>
+      </c>
+      <c r="C121" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B122" t="s">
-        <v>288</v>
+        <v>286</v>
+      </c>
+      <c r="C122" t="s">
+        <v>429</v>
+      </c>
+      <c r="D122" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B123" t="s">
-        <v>290</v>
+        <v>288</v>
+      </c>
+      <c r="C123" t="s">
+        <v>423</v>
+      </c>
+      <c r="D123" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B124" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C124" t="s">
-        <v>293</v>
+        <v>425</v>
       </c>
       <c r="D124" t="s">
-        <v>40</v>
+        <v>427</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B125" t="s">
-        <v>295</v>
+        <v>292</v>
+      </c>
+      <c r="C125" t="s">
+        <v>293</v>
+      </c>
+      <c r="D125" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>296</v>
-      </c>
       <c r="B126" t="s">
-        <v>297</v>
+        <v>421</v>
       </c>
       <c r="C126" t="s">
-        <v>298</v>
+        <v>426</v>
       </c>
       <c r="D126" t="s">
-        <v>58</v>
+        <v>427</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B127" t="s">
-        <v>300</v>
+        <v>419</v>
+      </c>
+      <c r="C127" t="s">
+        <v>424</v>
+      </c>
+      <c r="D127" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="B128" t="s">
-        <v>302</v>
+        <v>296</v>
+      </c>
+      <c r="C128" t="s">
+        <v>297</v>
+      </c>
+      <c r="D128" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="B129" t="s">
-        <v>304</v>
+        <v>299</v>
+      </c>
+      <c r="C129" t="s">
+        <v>428</v>
+      </c>
+      <c r="D129" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="B130" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="B131" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="B132" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B133" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="B134" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B135" t="s">
-        <v>316</v>
-      </c>
-      <c r="C135" t="s">
-        <v>217</v>
-      </c>
-      <c r="D135" t="s">
-        <v>218</v>
+        <v>311</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="B136" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="B137" t="s">
-        <v>320</v>
+        <v>315</v>
+      </c>
+      <c r="C137" t="s">
+        <v>217</v>
+      </c>
+      <c r="D137" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="B138" t="s">
-        <v>322</v>
-      </c>
-      <c r="C138" t="s">
-        <v>186</v>
-      </c>
-      <c r="D138" t="s">
-        <v>23</v>
+        <v>317</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="B139" t="s">
-        <v>324</v>
-      </c>
-      <c r="C139" t="s">
-        <v>327</v>
-      </c>
-      <c r="D139" t="s">
-        <v>23</v>
+        <v>319</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B140" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="C140" t="s">
-        <v>22</v>
+        <v>186</v>
       </c>
       <c r="D140" t="s">
         <v>23</v>
@@ -3085,362 +3136,368 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="B141" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="C141" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="D141" t="s">
-        <v>68</v>
+        <v>23</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="B142" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="C142" t="s">
-        <v>333</v>
+        <v>22</v>
       </c>
       <c r="D142" t="s">
-        <v>218</v>
+        <v>23</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="B143" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="C143" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="D143" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="B144" t="s">
-        <v>338</v>
+        <v>331</v>
+      </c>
+      <c r="C144" t="s">
+        <v>332</v>
+      </c>
+      <c r="D144" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="B145" t="s">
-        <v>340</v>
+        <v>334</v>
+      </c>
+      <c r="C145" t="s">
+        <v>335</v>
+      </c>
+      <c r="D145" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="B146" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="B147" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="B148" t="s">
-        <v>346</v>
-      </c>
-      <c r="C148" t="s">
-        <v>347</v>
-      </c>
-      <c r="D148" t="s">
-        <v>9</v>
+        <v>341</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
       <c r="B149" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="B150" t="s">
-        <v>351</v>
+        <v>345</v>
+      </c>
+      <c r="C150" t="s">
+        <v>346</v>
+      </c>
+      <c r="D150" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="B151" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B152" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="B153" t="s">
-        <v>357</v>
-      </c>
-      <c r="C153" t="s">
-        <v>358</v>
-      </c>
-      <c r="D153" t="s">
-        <v>23</v>
+        <v>352</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="B154" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="B155" t="s">
-        <v>362</v>
+        <v>356</v>
+      </c>
+      <c r="C155" t="s">
+        <v>357</v>
+      </c>
+      <c r="D155" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="B156" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="B157" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="B158" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B159" t="s">
-        <v>370</v>
-      </c>
-      <c r="C159" t="s">
-        <v>12</v>
-      </c>
-      <c r="D159" t="s">
-        <v>13</v>
+        <v>365</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="B160" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="B161" t="s">
-        <v>374</v>
+        <v>369</v>
+      </c>
+      <c r="C161" t="s">
+        <v>12</v>
+      </c>
+      <c r="D161" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="B162" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B163" t="s">
-        <v>378</v>
-      </c>
-      <c r="C163" t="s">
-        <v>139</v>
-      </c>
-      <c r="D163" t="s">
-        <v>58</v>
+        <v>373</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="B164" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="B165" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="C165" t="s">
-        <v>383</v>
+        <v>139</v>
       </c>
       <c r="D165" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="B166" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="B167" t="s">
-        <v>387</v>
+        <v>381</v>
+      </c>
+      <c r="C167" t="s">
+        <v>382</v>
+      </c>
+      <c r="D167" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="B168" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="B169" t="s">
-        <v>391</v>
-      </c>
-      <c r="C169" t="s">
-        <v>12</v>
-      </c>
-      <c r="D169" t="s">
-        <v>13</v>
+        <v>386</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="B170" t="s">
-        <v>393</v>
-      </c>
-      <c r="C170" t="s">
-        <v>12</v>
-      </c>
-      <c r="D170" t="s">
-        <v>13</v>
+        <v>388</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="B171" t="s">
-        <v>395</v>
+        <v>390</v>
+      </c>
+      <c r="C171" t="s">
+        <v>12</v>
+      </c>
+      <c r="D171" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B172" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="C172" t="s">
-        <v>398</v>
+        <v>12</v>
       </c>
       <c r="D172" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B173" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="B174" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="C174" t="s">
-        <v>12</v>
+        <v>397</v>
       </c>
       <c r="D174" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="B175" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="B176" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="C176" t="s">
         <v>12</v>
@@ -3451,60 +3508,82 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="B177" t="s">
-        <v>408</v>
-      </c>
-      <c r="C177" t="s">
-        <v>409</v>
-      </c>
-      <c r="D177" t="s">
-        <v>58</v>
+        <v>403</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="B178" t="s">
-        <v>411</v>
+        <v>405</v>
+      </c>
+      <c r="C178" t="s">
+        <v>12</v>
+      </c>
+      <c r="D178" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="B179" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="C179" t="s">
-        <v>12</v>
+        <v>408</v>
       </c>
       <c r="D179" t="s">
-        <v>13</v>
+        <v>58</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="B180" t="s">
-        <v>415</v>
-      </c>
-      <c r="C180" t="s">
-        <v>416</v>
-      </c>
-      <c r="D180" t="s">
-        <v>23</v>
+        <v>410</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
+        <v>411</v>
+      </c>
+      <c r="B181" t="s">
+        <v>412</v>
+      </c>
+      <c r="C181" t="s">
+        <v>12</v>
+      </c>
+      <c r="D181" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>413</v>
+      </c>
+      <c r="B182" t="s">
+        <v>414</v>
+      </c>
+      <c r="C182" t="s">
+        <v>415</v>
+      </c>
+      <c r="D182" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>416</v>
+      </c>
+      <c r="B183" t="s">
         <v>417</v>
-      </c>
-      <c r="B181" t="s">
-        <v>418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added 7 more opponents to verdant forest
</commit_message>
<xml_diff>
--- a/Coin_tracker.xlsx
+++ b/Coin_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C7951E-B1C6-47D3-A167-7DE97DA28B99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C5CB2A-BA71-41E7-9FD5-28079CC68554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="23385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="437">
   <si>
     <t>Coin</t>
   </si>
@@ -64,12 +64,6 @@
     <t>Day 3+</t>
   </si>
   <si>
-    <t>coin_back_basic.png</t>
-  </si>
-  <si>
-    <t>back basic</t>
-  </si>
-  <si>
     <t>coin_blastoise_blue.png</t>
   </si>
   <si>
@@ -439,9 +433,6 @@
     <t>energy green 2</t>
   </si>
   <si>
-    <t>BUG CATCHER JOHNNY</t>
-  </si>
-  <si>
     <t>coin_energy_pink.png</t>
   </si>
   <si>
@@ -1310,6 +1301,36 @@
   </si>
   <si>
     <t>Pikachu Mum</t>
+  </si>
+  <si>
+    <t>AROMA LADY PENELOPE</t>
+  </si>
+  <si>
+    <t>FOSSIL EXPERT JONATHAN</t>
+  </si>
+  <si>
+    <t>pokeball blue</t>
+  </si>
+  <si>
+    <t>pokeball gold</t>
+  </si>
+  <si>
+    <t>WISHING COIN GIVER</t>
+  </si>
+  <si>
+    <t>YOUNGSTER MILO</t>
+  </si>
+  <si>
+    <t>NINJABOY SASUKE</t>
+  </si>
+  <si>
+    <t>CARD EXPERT NATHAN</t>
+  </si>
+  <si>
+    <t>CARD EXPERT RUBY</t>
+  </si>
+  <si>
+    <t>SWIMMER BIBI</t>
   </si>
 </sst>
 </file>
@@ -1391,10 +1412,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D183" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:D183" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:D181">
-    <sortCondition ref="C1:C183"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D184" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D184" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D184">
+    <sortCondition ref="C1:C184"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Coin"/>
@@ -1723,7 +1744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D183"/>
+  <dimension ref="A1:D184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" hidden="1" customWidth="1"/>
@@ -1748,1842 +1769,1874 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>324</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>325</v>
+      </c>
+      <c r="C2" t="s">
+        <v>326</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>415</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>119</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>120</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>248</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>249</v>
+      </c>
+      <c r="C5" t="s">
+        <v>250</v>
+      </c>
+      <c r="D5" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>292</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>293</v>
+      </c>
+      <c r="C6" t="s">
+        <v>294</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>227</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>228</v>
+      </c>
+      <c r="C7" t="s">
+        <v>229</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>54</v>
+      </c>
+      <c r="C8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>132</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>133</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>178</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>179</v>
+      </c>
+      <c r="C10" t="s">
+        <v>180</v>
+      </c>
+      <c r="D10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>135</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" t="s">
-        <v>33</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>373</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>374</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>427</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>319</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>320</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>323</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>41</v>
+        <v>321</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>322</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>317</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>318</v>
+      </c>
+      <c r="C15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D15" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>176</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>177</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>49</v>
+        <v>201</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>202</v>
+      </c>
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>280</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>281</v>
+      </c>
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>53</v>
+        <v>365</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>366</v>
+      </c>
+      <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>55</v>
+        <v>386</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>387</v>
       </c>
       <c r="C21" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="D21" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>59</v>
+        <v>388</v>
       </c>
       <c r="B22" t="s">
-        <v>60</v>
+        <v>389</v>
+      </c>
+      <c r="C22" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>397</v>
       </c>
       <c r="B23" t="s">
-        <v>62</v>
+        <v>398</v>
+      </c>
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>63</v>
+        <v>401</v>
       </c>
       <c r="B24" t="s">
-        <v>64</v>
+        <v>402</v>
       </c>
       <c r="C24" t="s">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>68</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>65</v>
+        <v>408</v>
       </c>
       <c r="B25" t="s">
-        <v>66</v>
+        <v>409</v>
       </c>
       <c r="C25" t="s">
-        <v>418</v>
+        <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>218</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
       <c r="B26" t="s">
-        <v>70</v>
+        <v>126</v>
+      </c>
+      <c r="C26" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>71</v>
+        <v>212</v>
       </c>
       <c r="B27" t="s">
-        <v>72</v>
+        <v>213</v>
+      </c>
+      <c r="C27" t="s">
+        <v>214</v>
+      </c>
+      <c r="D27" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>73</v>
+        <v>311</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>312</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>75</v>
+        <v>144</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>145</v>
+      </c>
+      <c r="C29" t="s">
+        <v>146</v>
+      </c>
+      <c r="D29" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>6</v>
       </c>
       <c r="B30" t="s">
-        <v>78</v>
+        <v>7</v>
+      </c>
+      <c r="C30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>79</v>
+        <v>192</v>
       </c>
       <c r="B31" t="s">
-        <v>80</v>
+        <v>193</v>
+      </c>
+      <c r="C31" t="s">
+        <v>194</v>
+      </c>
+      <c r="D31" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>195</v>
       </c>
       <c r="B32" t="s">
-        <v>82</v>
+        <v>196</v>
+      </c>
+      <c r="C32" t="s">
+        <v>197</v>
+      </c>
+      <c r="D32" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>198</v>
       </c>
       <c r="B33" t="s">
-        <v>84</v>
+        <v>199</v>
+      </c>
+      <c r="C33" t="s">
+        <v>200</v>
+      </c>
+      <c r="D33" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>85</v>
+        <v>288</v>
       </c>
       <c r="B34" t="s">
-        <v>86</v>
+        <v>289</v>
+      </c>
+      <c r="C34" t="s">
+        <v>290</v>
+      </c>
+      <c r="D34" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>87</v>
+        <v>392</v>
       </c>
       <c r="B35" t="s">
-        <v>88</v>
+        <v>393</v>
+      </c>
+      <c r="C35" t="s">
+        <v>394</v>
+      </c>
+      <c r="D35" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="C36" t="s">
-        <v>91</v>
+        <v>24</v>
       </c>
       <c r="D36" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>92</v>
+        <v>352</v>
       </c>
       <c r="B37" t="s">
-        <v>93</v>
+        <v>353</v>
+      </c>
+      <c r="C37" t="s">
+        <v>354</v>
+      </c>
+      <c r="D37" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>94</v>
+        <v>410</v>
       </c>
       <c r="B38" t="s">
-        <v>95</v>
+        <v>411</v>
+      </c>
+      <c r="C38" t="s">
+        <v>412</v>
+      </c>
+      <c r="D38" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>96</v>
+        <v>377</v>
       </c>
       <c r="B39" t="s">
-        <v>97</v>
+        <v>378</v>
+      </c>
+      <c r="C39" t="s">
+        <v>379</v>
+      </c>
+      <c r="D39" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>98</v>
+        <v>267</v>
       </c>
       <c r="B40" t="s">
-        <v>99</v>
+        <v>268</v>
+      </c>
+      <c r="C40" t="s">
+        <v>269</v>
+      </c>
+      <c r="D40" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>100</v>
+        <v>341</v>
       </c>
       <c r="B41" t="s">
-        <v>101</v>
+        <v>342</v>
+      </c>
+      <c r="C41" t="s">
+        <v>343</v>
+      </c>
+      <c r="D41" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>102</v>
+        <v>257</v>
       </c>
       <c r="B42" t="s">
-        <v>103</v>
+        <v>258</v>
+      </c>
+      <c r="C42" t="s">
+        <v>259</v>
+      </c>
+      <c r="D42" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>104</v>
+        <v>261</v>
       </c>
       <c r="B43" t="s">
-        <v>105</v>
+        <v>262</v>
+      </c>
+      <c r="C43" t="s">
+        <v>259</v>
+      </c>
+      <c r="D43" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" t="s">
+        <v>105</v>
+      </c>
+      <c r="C44" t="s">
         <v>106</v>
       </c>
-      <c r="B44" t="s">
-        <v>107</v>
-      </c>
-      <c r="C44" t="s">
-        <v>108</v>
-      </c>
       <c r="D44" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>109</v>
+        <v>284</v>
       </c>
       <c r="B45" t="s">
-        <v>110</v>
+        <v>285</v>
+      </c>
+      <c r="C45" t="s">
+        <v>420</v>
+      </c>
+      <c r="D45" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>111</v>
+        <v>286</v>
       </c>
       <c r="B46" t="s">
-        <v>112</v>
+        <v>287</v>
+      </c>
+      <c r="C46" t="s">
+        <v>422</v>
+      </c>
+      <c r="D46" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>113</v>
-      </c>
       <c r="B47" t="s">
-        <v>114</v>
+        <v>417</v>
+      </c>
+      <c r="C47" t="s">
+        <v>419</v>
+      </c>
+      <c r="D47" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>115</v>
+        <v>295</v>
       </c>
       <c r="B48" t="s">
-        <v>116</v>
+        <v>296</v>
       </c>
       <c r="C48" t="s">
-        <v>117</v>
+        <v>425</v>
       </c>
       <c r="D48" t="s">
-        <v>58</v>
+        <v>424</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>118</v>
+        <v>291</v>
       </c>
       <c r="B49" t="s">
-        <v>119</v>
+        <v>416</v>
       </c>
       <c r="C49" t="s">
-        <v>120</v>
+        <v>421</v>
       </c>
       <c r="D49" t="s">
-        <v>58</v>
+        <v>424</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>121</v>
+        <v>282</v>
       </c>
       <c r="B50" t="s">
-        <v>122</v>
+        <v>283</v>
       </c>
       <c r="C50" t="s">
-        <v>123</v>
+        <v>426</v>
       </c>
       <c r="D50" t="s">
-        <v>58</v>
+        <v>424</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>124</v>
-      </c>
       <c r="B51" t="s">
-        <v>125</v>
+        <v>418</v>
       </c>
       <c r="C51" t="s">
-        <v>126</v>
+        <v>423</v>
       </c>
       <c r="D51" t="s">
-        <v>58</v>
+        <v>424</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="B52" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="C52" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="D52" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>130</v>
+        <v>327</v>
       </c>
       <c r="B53" t="s">
-        <v>131</v>
+        <v>328</v>
+      </c>
+      <c r="C53" t="s">
+        <v>329</v>
+      </c>
+      <c r="D53" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>132</v>
+        <v>330</v>
       </c>
       <c r="B54" t="s">
-        <v>133</v>
+        <v>331</v>
+      </c>
+      <c r="C54" t="s">
+        <v>332</v>
+      </c>
+      <c r="D54" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B55" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="C55" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="D55" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>137</v>
+        <v>35</v>
       </c>
       <c r="B56" t="s">
-        <v>138</v>
+        <v>36</v>
       </c>
       <c r="C56" t="s">
-        <v>139</v>
+        <v>37</v>
       </c>
       <c r="D56" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>140</v>
+        <v>205</v>
       </c>
       <c r="B57" t="s">
-        <v>141</v>
+        <v>206</v>
+      </c>
+      <c r="C57" t="s">
+        <v>207</v>
+      </c>
+      <c r="D57" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>142</v>
+        <v>87</v>
       </c>
       <c r="B58" t="s">
-        <v>143</v>
+        <v>88</v>
       </c>
       <c r="C58" t="s">
-        <v>144</v>
+        <v>89</v>
       </c>
       <c r="D58" t="s">
-        <v>68</v>
+        <v>31</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>145</v>
+        <v>403</v>
       </c>
       <c r="B59" t="s">
-        <v>146</v>
+        <v>404</v>
+      </c>
+      <c r="C59" t="s">
+        <v>405</v>
+      </c>
+      <c r="D59" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>147</v>
+        <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>148</v>
+        <v>62</v>
       </c>
       <c r="C60" t="s">
-        <v>149</v>
+        <v>65</v>
       </c>
       <c r="D60" t="s">
-        <v>9</v>
+        <v>66</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>150</v>
+        <v>113</v>
       </c>
       <c r="B61" t="s">
-        <v>151</v>
+        <v>114</v>
+      </c>
+      <c r="C61" t="s">
+        <v>115</v>
+      </c>
+      <c r="D61" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>152</v>
+        <v>216</v>
       </c>
       <c r="B62" t="s">
-        <v>153</v>
+        <v>217</v>
+      </c>
+      <c r="C62" t="s">
+        <v>218</v>
+      </c>
+      <c r="D62" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>154</v>
+        <v>116</v>
       </c>
       <c r="B63" t="s">
-        <v>155</v>
+        <v>117</v>
       </c>
       <c r="C63" t="s">
-        <v>156</v>
+        <v>118</v>
       </c>
       <c r="D63" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>157</v>
+        <v>28</v>
       </c>
       <c r="B64" t="s">
-        <v>158</v>
+        <v>29</v>
+      </c>
+      <c r="C64" t="s">
+        <v>30</v>
+      </c>
+      <c r="D64" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>159</v>
+        <v>32</v>
       </c>
       <c r="B65" t="s">
-        <v>160</v>
+        <v>33</v>
+      </c>
+      <c r="C65" t="s">
+        <v>34</v>
+      </c>
+      <c r="D65" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B66" t="s">
-        <v>162</v>
+        <v>152</v>
+      </c>
+      <c r="C66" t="s">
+        <v>153</v>
+      </c>
+      <c r="D66" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>163</v>
+        <v>4</v>
       </c>
       <c r="B67" t="s">
-        <v>164</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>165</v>
+        <v>14</v>
       </c>
       <c r="B68" t="s">
-        <v>166</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>167</v>
+        <v>16</v>
       </c>
       <c r="B69" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>169</v>
+        <v>18</v>
       </c>
       <c r="B70" t="s">
-        <v>170</v>
+        <v>19</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>171</v>
+        <v>26</v>
       </c>
       <c r="B71" t="s">
-        <v>172</v>
+        <v>27</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>173</v>
+        <v>39</v>
       </c>
       <c r="B72" t="s">
-        <v>174</v>
+        <v>40</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>175</v>
+        <v>41</v>
       </c>
       <c r="B73" t="s">
-        <v>176</v>
+        <v>42</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>177</v>
+        <v>43</v>
       </c>
       <c r="B74" t="s">
-        <v>178</v>
+        <v>44</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>179</v>
+        <v>45</v>
       </c>
       <c r="B75" t="s">
-        <v>180</v>
-      </c>
-      <c r="C75" t="s">
-        <v>12</v>
-      </c>
-      <c r="D75" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>181</v>
+        <v>47</v>
       </c>
       <c r="B76" t="s">
-        <v>182</v>
-      </c>
-      <c r="C76" t="s">
-        <v>183</v>
-      </c>
-      <c r="D76" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>184</v>
+        <v>49</v>
       </c>
       <c r="B77" t="s">
-        <v>185</v>
+        <v>50</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>187</v>
+        <v>51</v>
       </c>
       <c r="B78" t="s">
-        <v>188</v>
+        <v>52</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>189</v>
+        <v>57</v>
       </c>
       <c r="B79" t="s">
-        <v>190</v>
+        <v>58</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>191</v>
+        <v>59</v>
       </c>
       <c r="B80" t="s">
-        <v>192</v>
+        <v>60</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>193</v>
+        <v>67</v>
       </c>
       <c r="B81" t="s">
-        <v>194</v>
+        <v>68</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>195</v>
+        <v>69</v>
       </c>
       <c r="B82" t="s">
-        <v>196</v>
-      </c>
-      <c r="C82" t="s">
-        <v>197</v>
-      </c>
-      <c r="D82" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>198</v>
+        <v>71</v>
       </c>
       <c r="B83" t="s">
-        <v>199</v>
-      </c>
-      <c r="C83" t="s">
-        <v>200</v>
-      </c>
-      <c r="D83" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>201</v>
+        <v>73</v>
       </c>
       <c r="B84" t="s">
-        <v>202</v>
-      </c>
-      <c r="C84" t="s">
-        <v>203</v>
-      </c>
-      <c r="D84" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>204</v>
+        <v>75</v>
       </c>
       <c r="B85" t="s">
-        <v>205</v>
-      </c>
-      <c r="C85" t="s">
-        <v>12</v>
-      </c>
-      <c r="D85" t="s">
-        <v>13</v>
+        <v>76</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>206</v>
+        <v>77</v>
       </c>
       <c r="B86" t="s">
-        <v>207</v>
+        <v>78</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>208</v>
+        <v>79</v>
       </c>
       <c r="B87" t="s">
-        <v>209</v>
-      </c>
-      <c r="C87" t="s">
-        <v>210</v>
-      </c>
-      <c r="D87" t="s">
-        <v>33</v>
+        <v>80</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>211</v>
+        <v>81</v>
       </c>
       <c r="B88" t="s">
-        <v>212</v>
+        <v>82</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>213</v>
+        <v>83</v>
       </c>
       <c r="B89" t="s">
-        <v>214</v>
+        <v>84</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>215</v>
+        <v>85</v>
       </c>
       <c r="B90" t="s">
-        <v>216</v>
-      </c>
-      <c r="C90" t="s">
-        <v>217</v>
-      </c>
-      <c r="D90" t="s">
-        <v>218</v>
+        <v>86</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>219</v>
+        <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>220</v>
-      </c>
-      <c r="C91" t="s">
-        <v>221</v>
-      </c>
-      <c r="D91" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>222</v>
+        <v>92</v>
       </c>
       <c r="B92" t="s">
-        <v>223</v>
+        <v>93</v>
+      </c>
+      <c r="C92" t="s">
+        <v>432</v>
+      </c>
+      <c r="D92" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>224</v>
+        <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>225</v>
+        <v>95</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>226</v>
+        <v>96</v>
       </c>
       <c r="B94" t="s">
-        <v>227</v>
+        <v>97</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>228</v>
+        <v>98</v>
       </c>
       <c r="B95" t="s">
-        <v>229</v>
+        <v>99</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="B96" t="s">
-        <v>231</v>
-      </c>
-      <c r="C96" t="s">
-        <v>232</v>
-      </c>
-      <c r="D96" t="s">
-        <v>33</v>
+        <v>101</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>233</v>
+        <v>102</v>
       </c>
       <c r="B97" t="s">
-        <v>234</v>
+        <v>103</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>235</v>
+        <v>107</v>
       </c>
       <c r="B98" t="s">
-        <v>236</v>
+        <v>108</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>237</v>
+        <v>109</v>
       </c>
       <c r="B99" t="s">
-        <v>238</v>
+        <v>110</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>239</v>
+        <v>111</v>
       </c>
       <c r="B100" t="s">
-        <v>240</v>
+        <v>112</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>241</v>
+        <v>128</v>
       </c>
       <c r="B101" t="s">
-        <v>242</v>
+        <v>129</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>243</v>
+        <v>130</v>
       </c>
       <c r="B102" t="s">
-        <v>244</v>
+        <v>131</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>245</v>
+        <v>137</v>
       </c>
       <c r="B103" t="s">
-        <v>246</v>
+        <v>138</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>247</v>
+        <v>142</v>
       </c>
       <c r="B104" t="s">
-        <v>248</v>
+        <v>143</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>249</v>
+        <v>147</v>
       </c>
       <c r="B105" t="s">
-        <v>250</v>
+        <v>148</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>251</v>
+        <v>149</v>
       </c>
       <c r="B106" t="s">
-        <v>252</v>
-      </c>
-      <c r="C106" t="s">
-        <v>253</v>
-      </c>
-      <c r="D106" t="s">
-        <v>58</v>
+        <v>150</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>254</v>
+        <v>154</v>
       </c>
       <c r="B107" t="s">
-        <v>255</v>
+        <v>155</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>256</v>
+        <v>156</v>
       </c>
       <c r="B108" t="s">
-        <v>257</v>
-      </c>
-      <c r="D108" t="s">
-        <v>33</v>
+        <v>157</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>258</v>
+        <v>158</v>
       </c>
       <c r="B109" t="s">
-        <v>259</v>
+        <v>159</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>260</v>
+        <v>160</v>
       </c>
       <c r="B110" t="s">
-        <v>261</v>
-      </c>
-      <c r="C110" t="s">
-        <v>262</v>
-      </c>
-      <c r="D110" t="s">
-        <v>263</v>
+        <v>161</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>264</v>
+        <v>162</v>
       </c>
       <c r="B111" t="s">
-        <v>265</v>
+        <v>163</v>
       </c>
       <c r="C111" t="s">
-        <v>262</v>
+        <v>435</v>
       </c>
       <c r="D111" t="s">
-        <v>263</v>
+        <v>424</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>266</v>
+        <v>164</v>
       </c>
       <c r="B112" t="s">
-        <v>267</v>
+        <v>165</v>
+      </c>
+      <c r="C112" t="s">
+        <v>428</v>
+      </c>
+      <c r="D112" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>268</v>
+        <v>166</v>
       </c>
       <c r="B113" t="s">
-        <v>269</v>
+        <v>167</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>270</v>
+        <v>168</v>
       </c>
       <c r="B114" t="s">
-        <v>271</v>
+        <v>169</v>
       </c>
       <c r="C114" t="s">
-        <v>272</v>
+        <v>433</v>
       </c>
       <c r="D114" t="s">
-        <v>9</v>
+        <v>424</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>273</v>
+        <v>170</v>
       </c>
       <c r="B115" t="s">
-        <v>274</v>
+        <v>171</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>275</v>
+        <v>172</v>
       </c>
       <c r="B116" t="s">
-        <v>276</v>
+        <v>173</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>277</v>
+        <v>174</v>
       </c>
       <c r="B117" t="s">
-        <v>278</v>
+        <v>175</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>279</v>
+        <v>181</v>
       </c>
       <c r="B118" t="s">
-        <v>280</v>
+        <v>182</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>281</v>
+        <v>184</v>
       </c>
       <c r="B119" t="s">
-        <v>282</v>
+        <v>185</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>283</v>
+        <v>186</v>
       </c>
       <c r="B120" t="s">
-        <v>284</v>
-      </c>
-      <c r="C120" t="s">
-        <v>12</v>
-      </c>
-      <c r="D120" t="s">
-        <v>13</v>
+        <v>187</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>188</v>
+      </c>
       <c r="B121" t="s">
-        <v>420</v>
-      </c>
-      <c r="C121" t="s">
-        <v>422</v>
+        <v>189</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>285</v>
+        <v>190</v>
       </c>
       <c r="B122" t="s">
-        <v>286</v>
-      </c>
-      <c r="C122" t="s">
-        <v>429</v>
-      </c>
-      <c r="D122" t="s">
-        <v>427</v>
+        <v>191</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>287</v>
+        <v>203</v>
       </c>
       <c r="B123" t="s">
-        <v>288</v>
-      </c>
-      <c r="C123" t="s">
-        <v>423</v>
-      </c>
-      <c r="D123" t="s">
-        <v>427</v>
+        <v>204</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>289</v>
+        <v>208</v>
       </c>
       <c r="B124" t="s">
-        <v>290</v>
-      </c>
-      <c r="C124" t="s">
-        <v>425</v>
-      </c>
-      <c r="D124" t="s">
-        <v>427</v>
+        <v>209</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>291</v>
+        <v>210</v>
       </c>
       <c r="B125" t="s">
-        <v>292</v>
-      </c>
-      <c r="C125" t="s">
-        <v>293</v>
-      </c>
-      <c r="D125" t="s">
-        <v>40</v>
+        <v>211</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>219</v>
+      </c>
       <c r="B126" t="s">
-        <v>421</v>
-      </c>
-      <c r="C126" t="s">
-        <v>426</v>
-      </c>
-      <c r="D126" t="s">
-        <v>427</v>
+        <v>220</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>294</v>
+        <v>221</v>
       </c>
       <c r="B127" t="s">
-        <v>419</v>
-      </c>
-      <c r="C127" t="s">
-        <v>424</v>
-      </c>
-      <c r="D127" t="s">
-        <v>427</v>
+        <v>222</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>295</v>
+        <v>223</v>
       </c>
       <c r="B128" t="s">
-        <v>296</v>
-      </c>
-      <c r="C128" t="s">
-        <v>297</v>
-      </c>
-      <c r="D128" t="s">
-        <v>58</v>
+        <v>224</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>298</v>
+        <v>225</v>
       </c>
       <c r="B129" t="s">
-        <v>299</v>
-      </c>
-      <c r="C129" t="s">
-        <v>428</v>
-      </c>
-      <c r="D129" t="s">
-        <v>427</v>
+        <v>226</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>300</v>
+        <v>230</v>
       </c>
       <c r="B130" t="s">
-        <v>301</v>
+        <v>231</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>302</v>
+        <v>232</v>
       </c>
       <c r="B131" t="s">
-        <v>303</v>
+        <v>233</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>304</v>
+        <v>234</v>
       </c>
       <c r="B132" t="s">
-        <v>305</v>
+        <v>235</v>
+      </c>
+      <c r="C132" t="s">
+        <v>434</v>
+      </c>
+      <c r="D132" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>306</v>
+        <v>236</v>
       </c>
       <c r="B133" t="s">
-        <v>307</v>
+        <v>237</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>308</v>
+        <v>238</v>
       </c>
       <c r="B134" t="s">
-        <v>309</v>
+        <v>239</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>310</v>
+        <v>240</v>
       </c>
       <c r="B135" t="s">
-        <v>311</v>
+        <v>241</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>312</v>
+        <v>242</v>
       </c>
       <c r="B136" t="s">
-        <v>313</v>
+        <v>243</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>314</v>
+        <v>244</v>
       </c>
       <c r="B137" t="s">
-        <v>315</v>
-      </c>
-      <c r="C137" t="s">
-        <v>217</v>
-      </c>
-      <c r="D137" t="s">
-        <v>218</v>
+        <v>245</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>316</v>
+        <v>246</v>
       </c>
       <c r="B138" t="s">
-        <v>317</v>
+        <v>247</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>318</v>
+        <v>251</v>
       </c>
       <c r="B139" t="s">
-        <v>319</v>
+        <v>252</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>320</v>
+        <v>253</v>
       </c>
       <c r="B140" t="s">
-        <v>321</v>
-      </c>
-      <c r="C140" t="s">
-        <v>186</v>
-      </c>
-      <c r="D140" t="s">
-        <v>23</v>
+        <v>254</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>322</v>
+        <v>255</v>
       </c>
       <c r="B141" t="s">
-        <v>323</v>
-      </c>
-      <c r="C141" t="s">
-        <v>326</v>
-      </c>
-      <c r="D141" t="s">
-        <v>23</v>
+        <v>256</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>324</v>
+        <v>263</v>
       </c>
       <c r="B142" t="s">
-        <v>325</v>
-      </c>
-      <c r="C142" t="s">
-        <v>22</v>
-      </c>
-      <c r="D142" t="s">
-        <v>23</v>
+        <v>264</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>327</v>
+        <v>265</v>
       </c>
       <c r="B143" t="s">
-        <v>328</v>
-      </c>
-      <c r="C143" t="s">
-        <v>329</v>
-      </c>
-      <c r="D143" t="s">
-        <v>68</v>
+        <v>266</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>330</v>
+        <v>270</v>
       </c>
       <c r="B144" t="s">
-        <v>331</v>
-      </c>
-      <c r="C144" t="s">
-        <v>332</v>
-      </c>
-      <c r="D144" t="s">
-        <v>218</v>
+        <v>271</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>333</v>
+        <v>272</v>
       </c>
       <c r="B145" t="s">
-        <v>334</v>
-      </c>
-      <c r="C145" t="s">
-        <v>335</v>
-      </c>
-      <c r="D145" t="s">
-        <v>218</v>
+        <v>273</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>336</v>
+        <v>274</v>
       </c>
       <c r="B146" t="s">
-        <v>337</v>
+        <v>275</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>338</v>
+        <v>276</v>
       </c>
       <c r="B147" t="s">
-        <v>339</v>
+        <v>277</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>340</v>
+        <v>278</v>
       </c>
       <c r="B148" t="s">
-        <v>341</v>
+        <v>279</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>342</v>
+        <v>297</v>
       </c>
       <c r="B149" t="s">
-        <v>343</v>
+        <v>298</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>344</v>
+        <v>299</v>
       </c>
       <c r="B150" t="s">
-        <v>345</v>
-      </c>
-      <c r="C150" t="s">
-        <v>346</v>
-      </c>
-      <c r="D150" t="s">
-        <v>9</v>
+        <v>300</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>347</v>
+        <v>301</v>
       </c>
       <c r="B151" t="s">
-        <v>348</v>
+        <v>302</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
-        <v>349</v>
-      </c>
       <c r="B152" t="s">
-        <v>350</v>
+        <v>429</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
-        <v>351</v>
-      </c>
       <c r="B153" t="s">
-        <v>352</v>
+        <v>430</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>353</v>
+        <v>303</v>
       </c>
       <c r="B154" t="s">
-        <v>354</v>
+        <v>304</v>
+      </c>
+      <c r="C154" t="s">
+        <v>431</v>
+      </c>
+      <c r="D154" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>355</v>
+        <v>305</v>
       </c>
       <c r="B155" t="s">
-        <v>356</v>
-      </c>
-      <c r="C155" t="s">
-        <v>357</v>
-      </c>
-      <c r="D155" t="s">
-        <v>23</v>
+        <v>306</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>358</v>
+        <v>307</v>
       </c>
       <c r="B156" t="s">
-        <v>359</v>
+        <v>308</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>360</v>
+        <v>309</v>
       </c>
       <c r="B157" t="s">
-        <v>361</v>
+        <v>310</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>362</v>
+        <v>313</v>
       </c>
       <c r="B158" t="s">
-        <v>363</v>
+        <v>314</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>364</v>
+        <v>315</v>
       </c>
       <c r="B159" t="s">
-        <v>365</v>
+        <v>316</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>366</v>
+        <v>333</v>
       </c>
       <c r="B160" t="s">
-        <v>367</v>
+        <v>334</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>368</v>
+        <v>335</v>
       </c>
       <c r="B161" t="s">
-        <v>369</v>
-      </c>
-      <c r="C161" t="s">
-        <v>12</v>
-      </c>
-      <c r="D161" t="s">
-        <v>13</v>
+        <v>336</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>370</v>
+        <v>337</v>
       </c>
       <c r="B162" t="s">
-        <v>371</v>
+        <v>338</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>372</v>
+        <v>339</v>
       </c>
       <c r="B163" t="s">
-        <v>373</v>
+        <v>340</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>374</v>
+        <v>344</v>
       </c>
       <c r="B164" t="s">
-        <v>375</v>
+        <v>345</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>376</v>
+        <v>346</v>
       </c>
       <c r="B165" t="s">
-        <v>377</v>
-      </c>
-      <c r="C165" t="s">
-        <v>139</v>
-      </c>
-      <c r="D165" t="s">
-        <v>58</v>
+        <v>347</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>378</v>
+        <v>348</v>
       </c>
       <c r="B166" t="s">
-        <v>379</v>
+        <v>349</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>380</v>
+        <v>350</v>
       </c>
       <c r="B167" t="s">
-        <v>381</v>
-      </c>
-      <c r="C167" t="s">
-        <v>382</v>
-      </c>
-      <c r="D167" t="s">
-        <v>23</v>
+        <v>351</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>383</v>
+        <v>355</v>
       </c>
       <c r="B168" t="s">
-        <v>384</v>
+        <v>356</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>385</v>
+        <v>357</v>
       </c>
       <c r="B169" t="s">
-        <v>386</v>
+        <v>358</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>387</v>
+        <v>359</v>
       </c>
       <c r="B170" t="s">
-        <v>388</v>
+        <v>360</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>389</v>
+        <v>361</v>
       </c>
       <c r="B171" t="s">
-        <v>390</v>
+        <v>362</v>
       </c>
       <c r="C171" t="s">
-        <v>12</v>
+        <v>436</v>
       </c>
       <c r="D171" t="s">
-        <v>13</v>
+        <v>424</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>391</v>
+        <v>363</v>
       </c>
       <c r="B172" t="s">
-        <v>392</v>
-      </c>
-      <c r="C172" t="s">
-        <v>12</v>
-      </c>
-      <c r="D172" t="s">
-        <v>13</v>
+        <v>364</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>393</v>
+        <v>367</v>
       </c>
       <c r="B173" t="s">
-        <v>394</v>
+        <v>368</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>395</v>
+        <v>369</v>
       </c>
       <c r="B174" t="s">
-        <v>396</v>
-      </c>
-      <c r="C174" t="s">
-        <v>397</v>
-      </c>
-      <c r="D174" t="s">
-        <v>23</v>
+        <v>370</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>398</v>
+        <v>371</v>
       </c>
       <c r="B175" t="s">
-        <v>399</v>
+        <v>372</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
+        <v>375</v>
+      </c>
+      <c r="B176" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>380</v>
+      </c>
+      <c r="B177" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>382</v>
+      </c>
+      <c r="B178" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>384</v>
+      </c>
+      <c r="B179" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>390</v>
+      </c>
+      <c r="B180" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>395</v>
+      </c>
+      <c r="B181" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>399</v>
+      </c>
+      <c r="B182" t="s">
         <v>400</v>
       </c>
-      <c r="B176" t="s">
-        <v>401</v>
-      </c>
-      <c r="C176" t="s">
-        <v>12</v>
-      </c>
-      <c r="D176" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A177" t="s">
-        <v>402</v>
-      </c>
-      <c r="B177" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A178" t="s">
-        <v>404</v>
-      </c>
-      <c r="B178" t="s">
-        <v>405</v>
-      </c>
-      <c r="C178" t="s">
-        <v>12</v>
-      </c>
-      <c r="D178" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A179" t="s">
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
         <v>406</v>
       </c>
-      <c r="B179" t="s">
+      <c r="B183" t="s">
         <v>407</v>
       </c>
-      <c r="C179" t="s">
-        <v>408</v>
-      </c>
-      <c r="D179" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A180" t="s">
-        <v>409</v>
-      </c>
-      <c r="B180" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A181" t="s">
-        <v>411</v>
-      </c>
-      <c r="B181" t="s">
-        <v>412</v>
-      </c>
-      <c r="C181" t="s">
-        <v>12</v>
-      </c>
-      <c r="D181" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A182" t="s">
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
         <v>413</v>
       </c>
-      <c r="B182" t="s">
+      <c r="B184" t="s">
         <v>414</v>
-      </c>
-      <c r="C182" t="s">
-        <v>415</v>
-      </c>
-      <c r="D182" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A183" t="s">
-        <v>416</v>
-      </c>
-      <c r="B183" t="s">
-        <v>417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added coin shop purchasing NPC in Celeste Harbour
</commit_message>
<xml_diff>
--- a/Coin_tracker.xlsx
+++ b/Coin_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C5CB2A-BA71-41E7-9FD5-28079CC68554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C2AFFC-C340-472F-A558-DDF6E171B8D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1769,55 +1769,55 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>324</v>
+        <v>373</v>
       </c>
       <c r="B2" t="s">
-        <v>325</v>
+        <v>374</v>
       </c>
       <c r="C2" t="s">
-        <v>326</v>
+        <v>427</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>324</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>325</v>
       </c>
       <c r="C3" t="s">
-        <v>415</v>
+        <v>326</v>
       </c>
       <c r="D3" t="s">
-        <v>215</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>119</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>120</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>121</v>
+        <v>415</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>248</v>
+        <v>119</v>
       </c>
       <c r="B5" t="s">
-        <v>249</v>
+        <v>120</v>
       </c>
       <c r="C5" t="s">
-        <v>250</v>
+        <v>121</v>
       </c>
       <c r="D5" t="s">
         <v>56</v>
@@ -1825,13 +1825,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>292</v>
+        <v>248</v>
       </c>
       <c r="B6" t="s">
-        <v>293</v>
+        <v>249</v>
       </c>
       <c r="C6" t="s">
-        <v>294</v>
+        <v>250</v>
       </c>
       <c r="D6" t="s">
         <v>56</v>
@@ -1839,41 +1839,41 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>227</v>
+        <v>292</v>
       </c>
       <c r="B7" t="s">
-        <v>228</v>
+        <v>293</v>
       </c>
       <c r="C7" t="s">
-        <v>229</v>
+        <v>294</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>227</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>228</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>229</v>
       </c>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>132</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>134</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
         <v>56</v>
@@ -1881,49 +1881,55 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>178</v>
+        <v>132</v>
       </c>
       <c r="B10" t="s">
-        <v>179</v>
+        <v>133</v>
       </c>
       <c r="C10" t="s">
-        <v>180</v>
+        <v>134</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="B11" t="s">
-        <v>136</v>
+        <v>179</v>
+      </c>
+      <c r="C11" t="s">
+        <v>180</v>
+      </c>
+      <c r="D11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>373</v>
+        <v>319</v>
       </c>
       <c r="B12" t="s">
-        <v>374</v>
+        <v>320</v>
       </c>
       <c r="C12" t="s">
-        <v>427</v>
+        <v>323</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B13" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C13" t="s">
-        <v>323</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
@@ -1931,13 +1937,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="B14" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C14" t="s">
-        <v>20</v>
+        <v>183</v>
       </c>
       <c r="D14" t="s">
         <v>21</v>
@@ -1945,38 +1951,38 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>317</v>
+        <v>234</v>
       </c>
       <c r="B15" t="s">
-        <v>318</v>
+        <v>235</v>
       </c>
       <c r="C15" t="s">
-        <v>183</v>
+        <v>434</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>424</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>162</v>
       </c>
       <c r="B16" t="s">
-        <v>11</v>
+        <v>163</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>435</v>
       </c>
       <c r="D16" t="s">
-        <v>13</v>
+        <v>424</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>176</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>177</v>
+        <v>11</v>
       </c>
       <c r="C17" t="s">
         <v>12</v>
@@ -1987,10 +1993,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>201</v>
+        <v>176</v>
       </c>
       <c r="B18" t="s">
-        <v>202</v>
+        <v>177</v>
       </c>
       <c r="C18" t="s">
         <v>12</v>
@@ -2001,10 +2007,10 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>280</v>
+        <v>201</v>
       </c>
       <c r="B19" t="s">
-        <v>281</v>
+        <v>202</v>
       </c>
       <c r="C19" t="s">
         <v>12</v>
@@ -2015,10 +2021,10 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>365</v>
+        <v>280</v>
       </c>
       <c r="B20" t="s">
-        <v>366</v>
+        <v>281</v>
       </c>
       <c r="C20" t="s">
         <v>12</v>
@@ -2029,10 +2035,10 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>386</v>
+        <v>365</v>
       </c>
       <c r="B21" t="s">
-        <v>387</v>
+        <v>366</v>
       </c>
       <c r="C21" t="s">
         <v>12</v>
@@ -2043,10 +2049,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B22" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -2057,10 +2063,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="B23" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="C23" t="s">
         <v>12</v>
@@ -2071,10 +2077,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="B24" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
@@ -2085,10 +2091,10 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="B25" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="C25" t="s">
         <v>12</v>
@@ -2099,38 +2105,44 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>125</v>
+        <v>408</v>
       </c>
       <c r="B26" t="s">
-        <v>126</v>
+        <v>409</v>
       </c>
       <c r="C26" t="s">
-        <v>127</v>
+        <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>212</v>
+        <v>125</v>
       </c>
       <c r="B27" t="s">
-        <v>213</v>
+        <v>126</v>
       </c>
       <c r="C27" t="s">
-        <v>214</v>
+        <v>127</v>
       </c>
       <c r="D27" t="s">
-        <v>215</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>311</v>
+        <v>212</v>
       </c>
       <c r="B28" t="s">
-        <v>312</v>
+        <v>213</v>
+      </c>
+      <c r="C28" t="s">
+        <v>214</v>
+      </c>
+      <c r="D28" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -2205,69 +2217,69 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>288</v>
+        <v>164</v>
       </c>
       <c r="B34" t="s">
-        <v>289</v>
+        <v>165</v>
       </c>
       <c r="C34" t="s">
-        <v>290</v>
+        <v>428</v>
       </c>
       <c r="D34" t="s">
-        <v>38</v>
+        <v>424</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>392</v>
+        <v>288</v>
       </c>
       <c r="B35" t="s">
-        <v>393</v>
+        <v>289</v>
       </c>
       <c r="C35" t="s">
-        <v>394</v>
+        <v>290</v>
       </c>
       <c r="D35" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>22</v>
+        <v>392</v>
       </c>
       <c r="B36" t="s">
-        <v>23</v>
+        <v>393</v>
       </c>
       <c r="C36" t="s">
-        <v>24</v>
+        <v>394</v>
       </c>
       <c r="D36" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>352</v>
+        <v>22</v>
       </c>
       <c r="B37" t="s">
-        <v>353</v>
+        <v>23</v>
       </c>
       <c r="C37" t="s">
-        <v>354</v>
+        <v>24</v>
       </c>
       <c r="D37" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>410</v>
+        <v>352</v>
       </c>
       <c r="B38" t="s">
-        <v>411</v>
+        <v>353</v>
       </c>
       <c r="C38" t="s">
-        <v>412</v>
+        <v>354</v>
       </c>
       <c r="D38" t="s">
         <v>21</v>
@@ -2275,13 +2287,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>377</v>
+        <v>410</v>
       </c>
       <c r="B39" t="s">
-        <v>378</v>
+        <v>411</v>
       </c>
       <c r="C39" t="s">
-        <v>379</v>
+        <v>412</v>
       </c>
       <c r="D39" t="s">
         <v>21</v>
@@ -2289,27 +2301,27 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>267</v>
+        <v>377</v>
       </c>
       <c r="B40" t="s">
-        <v>268</v>
+        <v>378</v>
       </c>
       <c r="C40" t="s">
-        <v>269</v>
+        <v>379</v>
       </c>
       <c r="D40" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>341</v>
+        <v>267</v>
       </c>
       <c r="B41" t="s">
-        <v>342</v>
+        <v>268</v>
       </c>
       <c r="C41" t="s">
-        <v>343</v>
+        <v>269</v>
       </c>
       <c r="D41" t="s">
         <v>9</v>
@@ -2317,24 +2329,24 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>257</v>
+        <v>341</v>
       </c>
       <c r="B42" t="s">
-        <v>258</v>
+        <v>342</v>
       </c>
       <c r="C42" t="s">
-        <v>259</v>
+        <v>343</v>
       </c>
       <c r="D42" t="s">
-        <v>260</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B43" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C43" t="s">
         <v>259</v>
@@ -2345,27 +2357,27 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>104</v>
+        <v>261</v>
       </c>
       <c r="B44" t="s">
-        <v>105</v>
+        <v>262</v>
       </c>
       <c r="C44" t="s">
-        <v>106</v>
+        <v>259</v>
       </c>
       <c r="D44" t="s">
-        <v>25</v>
+        <v>260</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>284</v>
+        <v>168</v>
       </c>
       <c r="B45" t="s">
-        <v>285</v>
+        <v>169</v>
       </c>
       <c r="C45" t="s">
-        <v>420</v>
+        <v>433</v>
       </c>
       <c r="D45" t="s">
         <v>424</v>
@@ -2373,24 +2385,27 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>286</v>
+        <v>104</v>
       </c>
       <c r="B46" t="s">
-        <v>287</v>
+        <v>105</v>
       </c>
       <c r="C46" t="s">
-        <v>422</v>
+        <v>106</v>
       </c>
       <c r="D46" t="s">
-        <v>424</v>
+        <v>25</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>284</v>
+      </c>
       <c r="B47" t="s">
-        <v>417</v>
+        <v>285</v>
       </c>
       <c r="C47" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D47" t="s">
         <v>424</v>
@@ -2398,27 +2413,24 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="B48" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="C48" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="D48" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>291</v>
-      </c>
       <c r="B49" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C49" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D49" t="s">
         <v>424</v>
@@ -2426,24 +2438,27 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
       <c r="B50" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="C50" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D50" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>291</v>
+      </c>
       <c r="B51" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C51" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D51" t="s">
         <v>424</v>
@@ -2451,139 +2466,136 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>139</v>
+        <v>282</v>
       </c>
       <c r="B52" t="s">
-        <v>140</v>
+        <v>283</v>
       </c>
       <c r="C52" t="s">
-        <v>141</v>
+        <v>426</v>
       </c>
       <c r="D52" t="s">
-        <v>66</v>
+        <v>424</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>327</v>
-      </c>
       <c r="B53" t="s">
-        <v>328</v>
+        <v>418</v>
       </c>
       <c r="C53" t="s">
-        <v>329</v>
+        <v>423</v>
       </c>
       <c r="D53" t="s">
-        <v>215</v>
+        <v>424</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>330</v>
+        <v>139</v>
       </c>
       <c r="B54" t="s">
-        <v>331</v>
+        <v>140</v>
       </c>
       <c r="C54" t="s">
-        <v>332</v>
+        <v>141</v>
       </c>
       <c r="D54" t="s">
-        <v>215</v>
+        <v>66</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>122</v>
+        <v>327</v>
       </c>
       <c r="B55" t="s">
-        <v>123</v>
+        <v>328</v>
       </c>
       <c r="C55" t="s">
-        <v>124</v>
+        <v>329</v>
       </c>
       <c r="D55" t="s">
-        <v>56</v>
+        <v>215</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>35</v>
+        <v>330</v>
       </c>
       <c r="B56" t="s">
-        <v>36</v>
+        <v>331</v>
       </c>
       <c r="C56" t="s">
-        <v>37</v>
+        <v>332</v>
       </c>
       <c r="D56" t="s">
-        <v>38</v>
+        <v>215</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>205</v>
+        <v>122</v>
       </c>
       <c r="B57" t="s">
-        <v>206</v>
+        <v>123</v>
       </c>
       <c r="C57" t="s">
-        <v>207</v>
+        <v>124</v>
       </c>
       <c r="D57" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="B58" t="s">
-        <v>88</v>
+        <v>36</v>
       </c>
       <c r="C58" t="s">
-        <v>89</v>
+        <v>37</v>
       </c>
       <c r="D58" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>403</v>
+        <v>205</v>
       </c>
       <c r="B59" t="s">
-        <v>404</v>
+        <v>206</v>
       </c>
       <c r="C59" t="s">
-        <v>405</v>
+        <v>207</v>
       </c>
       <c r="D59" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="B60" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="C60" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="D60" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>113</v>
+        <v>403</v>
       </c>
       <c r="B61" t="s">
-        <v>114</v>
+        <v>404</v>
       </c>
       <c r="C61" t="s">
-        <v>115</v>
+        <v>405</v>
       </c>
       <c r="D61" t="s">
         <v>56</v>
@@ -2591,55 +2603,55 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>216</v>
+        <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>217</v>
+        <v>62</v>
       </c>
       <c r="C62" t="s">
-        <v>218</v>
+        <v>65</v>
       </c>
       <c r="D62" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>116</v>
+        <v>361</v>
       </c>
       <c r="B63" t="s">
-        <v>117</v>
+        <v>362</v>
       </c>
       <c r="C63" t="s">
-        <v>118</v>
+        <v>436</v>
       </c>
       <c r="D63" t="s">
-        <v>56</v>
+        <v>424</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>28</v>
+        <v>113</v>
       </c>
       <c r="B64" t="s">
-        <v>29</v>
+        <v>114</v>
       </c>
       <c r="C64" t="s">
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="D64" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>32</v>
+        <v>216</v>
       </c>
       <c r="B65" t="s">
-        <v>33</v>
+        <v>217</v>
       </c>
       <c r="C65" t="s">
-        <v>34</v>
+        <v>218</v>
       </c>
       <c r="D65" t="s">
         <v>31</v>
@@ -2647,895 +2659,883 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>151</v>
+        <v>116</v>
       </c>
       <c r="B66" t="s">
-        <v>152</v>
+        <v>117</v>
       </c>
       <c r="C66" t="s">
-        <v>153</v>
+        <v>118</v>
       </c>
       <c r="D66" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>4</v>
+        <v>303</v>
       </c>
       <c r="B67" t="s">
-        <v>5</v>
+        <v>304</v>
+      </c>
+      <c r="C67" t="s">
+        <v>431</v>
+      </c>
+      <c r="D67" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="B68" t="s">
-        <v>15</v>
+        <v>29</v>
+      </c>
+      <c r="C68" t="s">
+        <v>30</v>
+      </c>
+      <c r="D68" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="B69" t="s">
-        <v>17</v>
+        <v>33</v>
+      </c>
+      <c r="C69" t="s">
+        <v>34</v>
+      </c>
+      <c r="D69" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>18</v>
+        <v>151</v>
       </c>
       <c r="B70" t="s">
-        <v>19</v>
+        <v>152</v>
+      </c>
+      <c r="C70" t="s">
+        <v>153</v>
+      </c>
+      <c r="D70" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="B71" t="s">
-        <v>27</v>
+        <v>93</v>
+      </c>
+      <c r="C71" t="s">
+        <v>432</v>
+      </c>
+      <c r="D71" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>39</v>
+        <v>135</v>
       </c>
       <c r="B72" t="s">
-        <v>40</v>
+        <v>136</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>41</v>
+        <v>311</v>
       </c>
       <c r="B73" t="s">
-        <v>42</v>
+        <v>312</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="B74" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="B75" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="B76" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="B77" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="B78" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="B79" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>41</v>
+      </c>
+      <c r="B80" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>43</v>
+      </c>
+      <c r="B81" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>45</v>
+      </c>
+      <c r="B82" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>47</v>
+      </c>
+      <c r="B83" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>49</v>
+      </c>
+      <c r="B84" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>51</v>
+      </c>
+      <c r="B85" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>57</v>
+      </c>
+      <c r="B86" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>59</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B87" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>67</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B88" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>69</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B89" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>71</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B90" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>73</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B91" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>75</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B92" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>77</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B93" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>79</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B94" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>81</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B95" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>83</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B96" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>85</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B97" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>90</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B98" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>92</v>
-      </c>
-      <c r="B92" t="s">
-        <v>93</v>
-      </c>
-      <c r="C92" t="s">
-        <v>432</v>
-      </c>
-      <c r="D92" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>94</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B99" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>96</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B100" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>98</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B101" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>100</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B102" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
         <v>102</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B103" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
         <v>107</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B104" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
         <v>109</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B105" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
         <v>111</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B106" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
         <v>128</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B107" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>130</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B108" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
         <v>137</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B109" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
         <v>142</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B110" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
         <v>147</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B111" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
         <v>149</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B112" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
         <v>154</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B113" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
         <v>156</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B114" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
         <v>158</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B115" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
         <v>160</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B116" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>162</v>
-      </c>
-      <c r="B111" t="s">
-        <v>163</v>
-      </c>
-      <c r="C111" t="s">
-        <v>435</v>
-      </c>
-      <c r="D111" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>164</v>
-      </c>
-      <c r="B112" t="s">
-        <v>165</v>
-      </c>
-      <c r="C112" t="s">
-        <v>428</v>
-      </c>
-      <c r="D112" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
         <v>166</v>
       </c>
-      <c r="B113" t="s">
+      <c r="B117" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>168</v>
-      </c>
-      <c r="B114" t="s">
-        <v>169</v>
-      </c>
-      <c r="C114" t="s">
-        <v>433</v>
-      </c>
-      <c r="D114" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
         <v>170</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B118" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
         <v>172</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B119" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
         <v>174</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B120" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
         <v>181</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B121" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
         <v>184</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B122" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
         <v>186</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B123" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
         <v>188</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B124" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
         <v>190</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B125" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
         <v>203</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B126" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
         <v>208</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B127" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
         <v>210</v>
       </c>
-      <c r="B125" t="s">
+      <c r="B128" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
         <v>219</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B129" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
         <v>221</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B130" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
         <v>223</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B131" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
         <v>225</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B132" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
         <v>230</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B133" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
         <v>232</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B134" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
-        <v>234</v>
-      </c>
-      <c r="B132" t="s">
-        <v>235</v>
-      </c>
-      <c r="C132" t="s">
-        <v>434</v>
-      </c>
-      <c r="D132" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
         <v>236</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B135" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
         <v>238</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B136" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
         <v>240</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B137" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
         <v>242</v>
       </c>
-      <c r="B136" t="s">
+      <c r="B138" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
         <v>244</v>
       </c>
-      <c r="B137" t="s">
+      <c r="B139" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
         <v>246</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B140" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
         <v>251</v>
       </c>
-      <c r="B139" t="s">
+      <c r="B141" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
         <v>253</v>
       </c>
-      <c r="B140" t="s">
+      <c r="B142" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
         <v>255</v>
       </c>
-      <c r="B141" t="s">
+      <c r="B143" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
         <v>263</v>
       </c>
-      <c r="B142" t="s">
+      <c r="B144" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
         <v>265</v>
       </c>
-      <c r="B143" t="s">
+      <c r="B145" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A144" t="s">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
         <v>270</v>
       </c>
-      <c r="B144" t="s">
+      <c r="B146" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
         <v>272</v>
       </c>
-      <c r="B145" t="s">
+      <c r="B147" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A146" t="s">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
         <v>274</v>
       </c>
-      <c r="B146" t="s">
+      <c r="B148" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A147" t="s">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
         <v>276</v>
       </c>
-      <c r="B147" t="s">
+      <c r="B149" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
         <v>278</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B150" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
         <v>297</v>
       </c>
-      <c r="B149" t="s">
+      <c r="B151" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
         <v>299</v>
       </c>
-      <c r="B150" t="s">
+      <c r="B152" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
         <v>301</v>
       </c>
-      <c r="B151" t="s">
+      <c r="B153" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B152" t="s">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B154" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B153" t="s">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B155" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A154" t="s">
-        <v>303</v>
-      </c>
-      <c r="B154" t="s">
-        <v>304</v>
-      </c>
-      <c r="C154" t="s">
-        <v>431</v>
-      </c>
-      <c r="D154" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A155" t="s">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
         <v>305</v>
       </c>
-      <c r="B155" t="s">
+      <c r="B156" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A156" t="s">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
         <v>307</v>
       </c>
-      <c r="B156" t="s">
+      <c r="B157" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A157" t="s">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
         <v>309</v>
       </c>
-      <c r="B157" t="s">
+      <c r="B158" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A158" t="s">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
         <v>313</v>
       </c>
-      <c r="B158" t="s">
+      <c r="B159" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A159" t="s">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
         <v>315</v>
       </c>
-      <c r="B159" t="s">
+      <c r="B160" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A160" t="s">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
         <v>333</v>
       </c>
-      <c r="B160" t="s">
+      <c r="B161" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A161" t="s">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
         <v>335</v>
       </c>
-      <c r="B161" t="s">
+      <c r="B162" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A162" t="s">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
         <v>337</v>
       </c>
-      <c r="B162" t="s">
+      <c r="B163" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A163" t="s">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
         <v>339</v>
       </c>
-      <c r="B163" t="s">
+      <c r="B164" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A164" t="s">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
         <v>344</v>
       </c>
-      <c r="B164" t="s">
+      <c r="B165" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A165" t="s">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
         <v>346</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B166" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A166" t="s">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
         <v>348</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B167" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A167" t="s">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
         <v>350</v>
       </c>
-      <c r="B167" t="s">
+      <c r="B168" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A168" t="s">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
         <v>355</v>
       </c>
-      <c r="B168" t="s">
+      <c r="B169" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A169" t="s">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
         <v>357</v>
       </c>
-      <c r="B169" t="s">
+      <c r="B170" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A170" t="s">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
         <v>359</v>
       </c>
-      <c r="B170" t="s">
+      <c r="B171" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A171" t="s">
-        <v>361</v>
-      </c>
-      <c r="B171" t="s">
-        <v>362</v>
-      </c>
-      <c r="C171" t="s">
-        <v>436</v>
-      </c>
-      <c r="D171" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>363</v>
       </c>
@@ -3543,7 +3543,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>367</v>
       </c>
@@ -3551,7 +3551,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>369</v>
       </c>
@@ -3559,7 +3559,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>371</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>375</v>
       </c>

</xml_diff>

<commit_message>
Added holo rare gamble shop
</commit_message>
<xml_diff>
--- a/Coin_tracker.xlsx
+++ b/Coin_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C2AFFC-C340-472F-A558-DDF6E171B8D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6ABC041-AA64-423B-B4E4-384B05AA8046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="447">
   <si>
     <t>Coin</t>
   </si>
@@ -1331,6 +1331,36 @@
   </si>
   <si>
     <t>SWIMMER BIBI</t>
+  </si>
+  <si>
+    <t>FOREST RANGER TUCKER</t>
+  </si>
+  <si>
+    <t>LADY FIONA</t>
+  </si>
+  <si>
+    <t>Backpacker Patrick</t>
+  </si>
+  <si>
+    <t>CARD EXPERT AURORA</t>
+  </si>
+  <si>
+    <t>Mad Scientist Leonard</t>
+  </si>
+  <si>
+    <t>HIKER WALTER</t>
+  </si>
+  <si>
+    <t>Evening 4</t>
+  </si>
+  <si>
+    <t>DOCTOR MORTIMOR</t>
+  </si>
+  <si>
+    <t>SHADY CHARACTER OWEN</t>
+  </si>
+  <si>
+    <t>Night 4</t>
   </si>
 </sst>
 </file>
@@ -2941,7 +2971,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>85</v>
       </c>
@@ -2949,7 +2979,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>90</v>
       </c>
@@ -2957,15 +2987,21 @@
         <v>91</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>94</v>
       </c>
       <c r="B99" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C99" t="s">
+        <v>439</v>
+      </c>
+      <c r="D99" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>96</v>
       </c>
@@ -2973,7 +3009,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>98</v>
       </c>
@@ -2981,7 +3017,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>100</v>
       </c>
@@ -2989,7 +3025,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>102</v>
       </c>
@@ -2997,7 +3033,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>107</v>
       </c>
@@ -3005,7 +3041,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>109</v>
       </c>
@@ -3013,7 +3049,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>111</v>
       </c>
@@ -3021,7 +3057,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>128</v>
       </c>
@@ -3029,7 +3065,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>130</v>
       </c>
@@ -3037,7 +3073,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>137</v>
       </c>
@@ -3045,7 +3081,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>142</v>
       </c>
@@ -3053,7 +3089,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>147</v>
       </c>
@@ -3061,7 +3097,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>149</v>
       </c>
@@ -3069,7 +3105,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>154</v>
       </c>
@@ -3077,7 +3113,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>156</v>
       </c>
@@ -3085,7 +3121,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>158</v>
       </c>
@@ -3093,7 +3129,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>160</v>
       </c>
@@ -3101,7 +3137,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>166</v>
       </c>
@@ -3109,7 +3145,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>170</v>
       </c>
@@ -3117,7 +3153,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>172</v>
       </c>
@@ -3125,7 +3161,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>174</v>
       </c>
@@ -3133,7 +3169,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>181</v>
       </c>
@@ -3141,23 +3177,35 @@
         <v>182</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>184</v>
       </c>
       <c r="B122" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C122" t="s">
+        <v>440</v>
+      </c>
+      <c r="D122" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>186</v>
       </c>
       <c r="B123" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C123" t="s">
+        <v>438</v>
+      </c>
+      <c r="D123" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>188</v>
       </c>
@@ -3165,7 +3213,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>190</v>
       </c>
@@ -3173,7 +3221,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>203</v>
       </c>
@@ -3181,7 +3229,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>208</v>
       </c>
@@ -3189,15 +3237,21 @@
         <v>209</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>210</v>
       </c>
       <c r="B128" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C128" t="s">
+        <v>445</v>
+      </c>
+      <c r="D128" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>219</v>
       </c>
@@ -3205,7 +3259,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>221</v>
       </c>
@@ -3213,7 +3267,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>223</v>
       </c>
@@ -3221,7 +3275,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>225</v>
       </c>
@@ -3229,7 +3283,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>230</v>
       </c>
@@ -3237,7 +3291,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>232</v>
       </c>
@@ -3245,7 +3299,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>236</v>
       </c>
@@ -3253,7 +3307,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>238</v>
       </c>
@@ -3261,7 +3315,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>240</v>
       </c>
@@ -3269,15 +3323,21 @@
         <v>241</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>242</v>
       </c>
       <c r="B138" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C138" t="s">
+        <v>441</v>
+      </c>
+      <c r="D138" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>244</v>
       </c>
@@ -3285,7 +3345,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>246</v>
       </c>
@@ -3293,7 +3353,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>251</v>
       </c>
@@ -3301,7 +3361,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>253</v>
       </c>
@@ -3309,7 +3369,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>255</v>
       </c>
@@ -3317,7 +3377,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>263</v>
       </c>
@@ -3447,7 +3507,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>333</v>
       </c>
@@ -3455,7 +3515,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>335</v>
       </c>
@@ -3463,7 +3523,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>337</v>
       </c>
@@ -3471,15 +3531,21 @@
         <v>338</v>
       </c>
     </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>339</v>
       </c>
       <c r="B164" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C164" t="s">
+        <v>437</v>
+      </c>
+      <c r="D164" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>344</v>
       </c>
@@ -3487,7 +3553,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>346</v>
       </c>
@@ -3495,7 +3561,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>348</v>
       </c>
@@ -3503,7 +3569,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>350</v>
       </c>
@@ -3511,7 +3577,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>355</v>
       </c>
@@ -3519,15 +3585,21 @@
         <v>356</v>
       </c>
     </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>357</v>
       </c>
       <c r="B170" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C170" t="s">
+        <v>442</v>
+      </c>
+      <c r="D170" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>359</v>
       </c>
@@ -3535,15 +3607,21 @@
         <v>360</v>
       </c>
     </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>363</v>
       </c>
       <c r="B172" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C172" t="s">
+        <v>444</v>
+      </c>
+      <c r="D172" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>367</v>
       </c>
@@ -3551,7 +3629,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>369</v>
       </c>
@@ -3559,7 +3637,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>371</v>
       </c>
@@ -3567,7 +3645,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>375</v>
       </c>

</xml_diff>